<commit_message>
Update deliveries and price data
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Myburgh Swiegers\Projects\Codex_GDI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E02AEF0-CFFA-4E21-A870-D29879B9D103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94606E6F-2876-4869-A967-5DC411C52669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2181" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2182" uniqueCount="730">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2223,6 +2223,9 @@
   </si>
   <si>
     <t>13/06 - 19/06/2026</t>
+  </si>
+  <si>
+    <t>20/06 - 26/06/2026</t>
   </si>
 </sst>
 </file>
@@ -2236,7 +2239,7 @@
     <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="#\ ###\ ##0"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2329,12 +2332,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="16">
@@ -2429,7 +2426,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -2639,13 +2636,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0A0101"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF0A0101"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color rgb="FF0A0101"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2764,14 +2774,15 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3145,11 +3156,11 @@
         <v>76</v>
       </c>
       <c r="AC1" s="45"/>
-      <c r="AD1" s="60" t="s">
+      <c r="AD1" s="58" t="s">
         <v>723</v>
       </c>
-      <c r="AE1" s="60"/>
-      <c r="AF1" s="61"/>
+      <c r="AE1" s="58"/>
+      <c r="AF1" s="59"/>
     </row>
     <row r="2" spans="1:32" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31">
@@ -56203,7 +56214,7 @@
       <c r="B680" s="18">
         <v>9</v>
       </c>
-      <c r="C680" s="44" t="s">
+      <c r="C680" s="60" t="s">
         <v>78</v>
       </c>
       <c r="D680" s="15" t="s">
@@ -56216,31 +56227,31 @@
         <v>28062</v>
       </c>
       <c r="G680" s="16">
-        <v>-23963</v>
+        <v>-24055</v>
       </c>
       <c r="H680" s="16">
-        <v>4099</v>
+        <v>4007</v>
       </c>
       <c r="I680" s="16">
         <v>67676</v>
       </c>
       <c r="J680" s="16">
-        <v>-57180</v>
+        <v>-58015</v>
       </c>
       <c r="K680" s="16">
-        <v>10496</v>
+        <v>9661</v>
       </c>
       <c r="L680" s="16">
         <v>95738</v>
       </c>
       <c r="M680" s="16">
-        <v>-81143</v>
+        <v>-82070</v>
       </c>
       <c r="N680" s="16">
-        <v>14595</v>
+        <v>13668</v>
       </c>
       <c r="O680" s="16">
-        <v>3669</v>
+        <v>3577</v>
       </c>
       <c r="P680" s="16">
         <v>429</v>
@@ -56252,10 +56263,10 @@
         <v>0</v>
       </c>
       <c r="S680" s="16">
-        <v>4099</v>
+        <v>4007</v>
       </c>
       <c r="T680" s="16">
-        <v>10373</v>
+        <v>9538</v>
       </c>
       <c r="U680" s="16">
         <v>123</v>
@@ -56267,10 +56278,10 @@
         <v>0</v>
       </c>
       <c r="X680" s="16">
-        <v>10496</v>
+        <v>9661</v>
       </c>
       <c r="Y680" s="16">
-        <v>14595</v>
+        <v>13668</v>
       </c>
       <c r="Z680" s="19"/>
       <c r="AA680" s="57"/>
@@ -56282,7 +56293,7 @@
       <c r="B681" s="4">
         <v>10</v>
       </c>
-      <c r="C681" s="8" t="s">
+      <c r="C681" s="61" t="s">
         <v>79</v>
       </c>
       <c r="D681" s="6" t="s">
@@ -56304,19 +56315,19 @@
         <v>73014</v>
       </c>
       <c r="J681" s="10">
-        <v>524</v>
+        <v>385</v>
       </c>
       <c r="K681" s="10">
-        <v>73538</v>
+        <v>73399</v>
       </c>
       <c r="L681" s="10">
         <v>102013</v>
       </c>
       <c r="M681" s="10">
-        <v>1000</v>
+        <v>861</v>
       </c>
       <c r="N681" s="10">
-        <v>103013</v>
+        <v>102874</v>
       </c>
       <c r="O681" s="10">
         <v>27608</v>
@@ -56334,7 +56345,7 @@
         <v>29475</v>
       </c>
       <c r="T681" s="10">
-        <v>72223</v>
+        <v>72084</v>
       </c>
       <c r="U681" s="10">
         <v>1182</v>
@@ -56346,10 +56357,10 @@
         <v>78</v>
       </c>
       <c r="X681" s="10">
-        <v>73538</v>
+        <v>73399</v>
       </c>
       <c r="Y681" s="10">
-        <v>103013</v>
+        <v>102874</v>
       </c>
       <c r="AA681" s="57"/>
     </row>
@@ -56360,7 +56371,7 @@
       <c r="B682" s="4">
         <v>11</v>
       </c>
-      <c r="C682" s="8" t="s">
+      <c r="C682" s="61" t="s">
         <v>80</v>
       </c>
       <c r="D682" s="6" t="s">
@@ -56382,19 +56393,19 @@
         <v>137597</v>
       </c>
       <c r="J682" s="10">
-        <v>2799</v>
+        <v>2480</v>
       </c>
       <c r="K682" s="10">
-        <v>140396</v>
+        <v>140077</v>
       </c>
       <c r="L682" s="10">
         <v>205271</v>
       </c>
       <c r="M682" s="10">
-        <v>2953</v>
+        <v>2634</v>
       </c>
       <c r="N682" s="10">
-        <v>208224</v>
+        <v>207905</v>
       </c>
       <c r="O682" s="10">
         <v>63822</v>
@@ -56412,7 +56423,7 @@
         <v>67828</v>
       </c>
       <c r="T682" s="10">
-        <v>137395</v>
+        <v>137076</v>
       </c>
       <c r="U682" s="10">
         <v>2859</v>
@@ -56424,10 +56435,10 @@
         <v>37</v>
       </c>
       <c r="X682" s="10">
-        <v>140396</v>
+        <v>140077</v>
       </c>
       <c r="Y682" s="10">
-        <v>208224</v>
+        <v>207905</v>
       </c>
       <c r="AA682" s="57"/>
     </row>
@@ -56438,7 +56449,7 @@
       <c r="B683" s="4">
         <v>12</v>
       </c>
-      <c r="C683" s="8" t="s">
+      <c r="C683" s="61" t="s">
         <v>81</v>
       </c>
       <c r="D683" s="6" t="s">
@@ -56451,31 +56462,31 @@
         <v>120859</v>
       </c>
       <c r="G683" s="10">
-        <v>774</v>
+        <v>-193</v>
       </c>
       <c r="H683" s="10">
-        <v>121633</v>
+        <v>120666</v>
       </c>
       <c r="I683" s="10">
         <v>285962</v>
       </c>
       <c r="J683" s="10">
-        <v>2233</v>
+        <v>2824</v>
       </c>
       <c r="K683" s="10">
-        <v>288195</v>
+        <v>288786</v>
       </c>
       <c r="L683" s="10">
         <v>406821</v>
       </c>
       <c r="M683" s="10">
-        <v>3007</v>
+        <v>2631</v>
       </c>
       <c r="N683" s="10">
-        <v>409828</v>
+        <v>409452</v>
       </c>
       <c r="O683" s="10">
-        <v>116586</v>
+        <v>115619</v>
       </c>
       <c r="P683" s="10">
         <v>4216</v>
@@ -56487,10 +56498,10 @@
         <v>111</v>
       </c>
       <c r="S683" s="10">
-        <v>121633</v>
+        <v>120666</v>
       </c>
       <c r="T683" s="10">
-        <v>276837</v>
+        <v>277428</v>
       </c>
       <c r="U683" s="10">
         <v>10777</v>
@@ -56502,10 +56513,10 @@
         <v>2</v>
       </c>
       <c r="X683" s="10">
-        <v>288195</v>
+        <v>288786</v>
       </c>
       <c r="Y683" s="10">
-        <v>409828</v>
+        <v>409452</v>
       </c>
       <c r="AA683" s="57"/>
     </row>
@@ -56516,7 +56527,7 @@
       <c r="B684" s="4">
         <v>13</v>
       </c>
-      <c r="C684" s="8" t="s">
+      <c r="C684" s="61" t="s">
         <v>82</v>
       </c>
       <c r="D684" s="6" t="s">
@@ -56529,31 +56540,31 @@
         <v>201415</v>
       </c>
       <c r="G684" s="10">
-        <v>7926</v>
+        <v>10982</v>
       </c>
       <c r="H684" s="10">
-        <v>209341</v>
+        <v>212397</v>
       </c>
       <c r="I684" s="10">
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>20940</v>
+        <v>32252</v>
       </c>
       <c r="K684" s="10">
-        <v>433799</v>
+        <v>445111</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>28866</v>
+        <v>43234</v>
       </c>
       <c r="N684" s="10">
-        <v>643140</v>
+        <v>657508</v>
       </c>
       <c r="O684" s="10">
-        <v>200424</v>
+        <v>203480</v>
       </c>
       <c r="P684" s="10">
         <v>8021</v>
@@ -56565,10 +56576,10 @@
         <v>135</v>
       </c>
       <c r="S684" s="10">
-        <v>209341</v>
+        <v>212397</v>
       </c>
       <c r="T684" s="10">
-        <v>410049</v>
+        <v>421361</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56580,10 +56591,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>433799</v>
+        <v>445111</v>
       </c>
       <c r="Y684" s="10">
-        <v>643140</v>
+        <v>657508</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56594,7 +56605,7 @@
       <c r="B685" s="4">
         <v>14</v>
       </c>
-      <c r="C685" s="8" t="s">
+      <c r="C685" s="61" t="s">
         <v>83</v>
       </c>
       <c r="D685" s="6" t="s">
@@ -56616,19 +56627,19 @@
         <v>435387</v>
       </c>
       <c r="J685" s="10">
-        <v>11482</v>
+        <v>12821</v>
       </c>
       <c r="K685" s="10">
-        <v>446869</v>
+        <v>448208</v>
       </c>
       <c r="L685" s="10">
         <v>726265</v>
       </c>
       <c r="M685" s="10">
-        <v>11849</v>
+        <v>13188</v>
       </c>
       <c r="N685" s="10">
-        <v>738114</v>
+        <v>739453</v>
       </c>
       <c r="O685" s="10">
         <v>274716</v>
@@ -56646,7 +56657,7 @@
         <v>291245</v>
       </c>
       <c r="T685" s="10">
-        <v>411169</v>
+        <v>412508</v>
       </c>
       <c r="U685" s="10">
         <v>34786</v>
@@ -56658,10 +56669,10 @@
         <v>48</v>
       </c>
       <c r="X685" s="10">
-        <v>446869</v>
+        <v>448208</v>
       </c>
       <c r="Y685" s="10">
-        <v>738114</v>
+        <v>739453</v>
       </c>
       <c r="AA685" s="57"/>
     </row>
@@ -56672,7 +56683,7 @@
       <c r="B686" s="4">
         <v>15</v>
       </c>
-      <c r="C686" s="58" t="s">
+      <c r="C686" s="61" t="s">
         <v>727</v>
       </c>
       <c r="D686" s="6" t="s">
@@ -56694,19 +56705,19 @@
         <v>592608</v>
       </c>
       <c r="J686" s="6">
-        <v>880</v>
+        <v>2409</v>
       </c>
       <c r="K686" s="6">
-        <v>593488</v>
+        <v>595017</v>
       </c>
       <c r="L686" s="6">
         <v>1110226</v>
       </c>
       <c r="M686" s="6">
-        <v>1611</v>
+        <v>3140</v>
       </c>
       <c r="N686" s="6">
-        <v>1111837</v>
+        <v>1113366</v>
       </c>
       <c r="O686" s="6">
         <v>490354</v>
@@ -56724,7 +56735,7 @@
         <v>518349</v>
       </c>
       <c r="T686" s="6">
-        <v>535776</v>
+        <v>537305</v>
       </c>
       <c r="U686" s="6">
         <v>54295</v>
@@ -56736,10 +56747,10 @@
         <v>189</v>
       </c>
       <c r="X686" s="6">
-        <v>593488</v>
+        <v>595017</v>
       </c>
       <c r="Y686" s="6">
-        <v>1111837</v>
+        <v>1113366</v>
       </c>
       <c r="AA686" s="57"/>
     </row>
@@ -56750,7 +56761,7 @@
       <c r="B687" s="4">
         <v>16</v>
       </c>
-      <c r="C687" s="59" t="s">
+      <c r="C687" s="61" t="s">
         <v>728</v>
       </c>
       <c r="D687" s="6" t="s">
@@ -56763,31 +56774,31 @@
         <v>702695</v>
       </c>
       <c r="G687" s="6">
-        <v>0</v>
+        <v>-35</v>
       </c>
       <c r="H687" s="6">
-        <v>702695</v>
+        <v>702660</v>
       </c>
       <c r="I687" s="6">
         <v>669414</v>
       </c>
       <c r="J687" s="6">
-        <v>0</v>
+        <v>1243</v>
       </c>
       <c r="K687" s="6">
-        <v>669414</v>
+        <v>670657</v>
       </c>
       <c r="L687" s="6">
         <v>1372109</v>
       </c>
       <c r="M687" s="6">
-        <v>0</v>
+        <v>1208</v>
       </c>
       <c r="N687" s="6">
-        <v>1372109</v>
+        <v>1373317</v>
       </c>
       <c r="O687" s="6">
-        <v>666238</v>
+        <v>666203</v>
       </c>
       <c r="P687" s="6">
         <v>34602</v>
@@ -56799,10 +56810,10 @@
         <v>45</v>
       </c>
       <c r="S687" s="6">
-        <v>702695</v>
+        <v>702660</v>
       </c>
       <c r="T687" s="6">
-        <v>608131</v>
+        <v>609374</v>
       </c>
       <c r="U687" s="6">
         <v>57879</v>
@@ -56814,10 +56825,10 @@
         <v>138</v>
       </c>
       <c r="X687" s="6">
-        <v>669414</v>
+        <v>670657</v>
       </c>
       <c r="Y687" s="6">
-        <v>1372109</v>
+        <v>1373317</v>
       </c>
     </row>
     <row r="688" spans="1:27" x14ac:dyDescent="0.25">
@@ -56827,33 +56838,75 @@
       <c r="B688" s="4">
         <v>17</v>
       </c>
-      <c r="C688" s="7"/>
+      <c r="C688" s="62" t="s">
+        <v>729</v>
+      </c>
       <c r="D688" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E688" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F688" s="6"/>
-      <c r="G688" s="6"/>
-      <c r="H688" s="6"/>
-      <c r="I688" s="6"/>
-      <c r="J688" s="6"/>
-      <c r="K688" s="6"/>
-      <c r="L688" s="6"/>
-      <c r="M688" s="6"/>
-      <c r="N688" s="6"/>
-      <c r="O688" s="6"/>
-      <c r="P688" s="6"/>
-      <c r="Q688" s="6"/>
-      <c r="R688" s="6"/>
-      <c r="S688" s="6"/>
-      <c r="T688" s="6"/>
-      <c r="U688" s="6"/>
-      <c r="V688" s="6"/>
-      <c r="W688" s="6"/>
-      <c r="X688" s="6"/>
-      <c r="Y688" s="6"/>
+      <c r="F688" s="6">
+        <v>456498</v>
+      </c>
+      <c r="G688" s="6">
+        <v>0</v>
+      </c>
+      <c r="H688" s="6">
+        <v>456498</v>
+      </c>
+      <c r="I688" s="6">
+        <v>390877</v>
+      </c>
+      <c r="J688" s="6">
+        <v>0</v>
+      </c>
+      <c r="K688" s="6">
+        <v>390877</v>
+      </c>
+      <c r="L688" s="6">
+        <v>847375</v>
+      </c>
+      <c r="M688" s="6">
+        <v>0</v>
+      </c>
+      <c r="N688" s="6">
+        <v>847375</v>
+      </c>
+      <c r="O688" s="6">
+        <v>429286</v>
+      </c>
+      <c r="P688" s="6">
+        <v>24519</v>
+      </c>
+      <c r="Q688" s="6">
+        <v>2657</v>
+      </c>
+      <c r="R688" s="6">
+        <v>36</v>
+      </c>
+      <c r="S688" s="6">
+        <v>456498</v>
+      </c>
+      <c r="T688" s="6">
+        <v>358493</v>
+      </c>
+      <c r="U688" s="6">
+        <v>31372</v>
+      </c>
+      <c r="V688" s="6">
+        <v>824</v>
+      </c>
+      <c r="W688" s="6">
+        <v>188</v>
+      </c>
+      <c r="X688" s="6">
+        <v>390877</v>
+      </c>
+      <c r="Y688" s="6">
+        <v>847375</v>
+      </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A689" s="7">
@@ -58350,26 +58403,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -58596,10 +58629,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
+    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -58616,20 +58680,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
-    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update AGR and CFTC data and maize import workflow
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Myburgh Swiegers\Projects\Codex_GDI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1C1A65-47F3-4F72-9060-CE69601FA763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E92842-B669-42CD-A72F-D1D679DE64B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28980" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2184" uniqueCount="732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2186" uniqueCount="734">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2232,6 +2232,12 @@
   </si>
   <si>
     <t>04/07 - 10/07/2026</t>
+  </si>
+  <si>
+    <t>11/07 - 17/07/2026</t>
+  </si>
+  <si>
+    <t>18/07 - 24/07/2026</t>
   </si>
 </sst>
 </file>
@@ -2245,7 +2251,7 @@
     <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="#\ ###\ ##0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2338,6 +2344,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Narrow"/>
     </font>
   </fonts>
   <fills count="16">
@@ -2786,9 +2797,9 @@
     <xf numFmtId="0" fontId="9" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -56336,13 +56347,13 @@
         <v>102874</v>
       </c>
       <c r="O681" s="10">
-        <v>27608</v>
+        <v>27562</v>
       </c>
       <c r="P681" s="10">
         <v>1766</v>
       </c>
       <c r="Q681" s="10">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="R681" s="10">
         <v>91</v>
@@ -56555,19 +56566,19 @@
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>32321</v>
+        <v>33866</v>
       </c>
       <c r="K684" s="10">
-        <v>445180</v>
+        <v>446725</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>43596</v>
+        <v>45141</v>
       </c>
       <c r="N684" s="10">
-        <v>657870</v>
+        <v>659415</v>
       </c>
       <c r="O684" s="10">
         <v>203773</v>
@@ -56585,7 +56596,7 @@
         <v>212690</v>
       </c>
       <c r="T684" s="10">
-        <v>421430</v>
+        <v>422975</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56597,10 +56608,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>445180</v>
+        <v>446725</v>
       </c>
       <c r="Y684" s="10">
-        <v>657870</v>
+        <v>659415</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56624,31 +56635,31 @@
         <v>290878</v>
       </c>
       <c r="G685" s="10">
-        <v>1536</v>
+        <v>1711</v>
       </c>
       <c r="H685" s="10">
-        <v>292414</v>
+        <v>292589</v>
       </c>
       <c r="I685" s="10">
         <v>435387</v>
       </c>
       <c r="J685" s="10">
-        <v>14241</v>
+        <v>15129</v>
       </c>
       <c r="K685" s="10">
-        <v>449628</v>
+        <v>450516</v>
       </c>
       <c r="L685" s="10">
         <v>726265</v>
       </c>
       <c r="M685" s="10">
-        <v>15777</v>
+        <v>16840</v>
       </c>
       <c r="N685" s="10">
-        <v>742042</v>
+        <v>743105</v>
       </c>
       <c r="O685" s="10">
-        <v>275885</v>
+        <v>276060</v>
       </c>
       <c r="P685" s="10">
         <v>15443</v>
@@ -56660,10 +56671,10 @@
         <v>69</v>
       </c>
       <c r="S685" s="10">
-        <v>292414</v>
+        <v>292589</v>
       </c>
       <c r="T685" s="10">
-        <v>413928</v>
+        <v>414816</v>
       </c>
       <c r="U685" s="10">
         <v>34786</v>
@@ -56675,10 +56686,10 @@
         <v>48</v>
       </c>
       <c r="X685" s="10">
-        <v>449628</v>
+        <v>450516</v>
       </c>
       <c r="Y685" s="10">
-        <v>742042</v>
+        <v>743105</v>
       </c>
       <c r="AA685" s="57"/>
     </row>
@@ -56702,31 +56713,31 @@
         <v>517618</v>
       </c>
       <c r="G686" s="6">
-        <v>6259</v>
+        <v>7338</v>
       </c>
       <c r="H686" s="6">
-        <v>523877</v>
+        <v>524956</v>
       </c>
       <c r="I686" s="6">
         <v>592608</v>
       </c>
       <c r="J686" s="6">
-        <v>3962</v>
+        <v>7187</v>
       </c>
       <c r="K686" s="6">
-        <v>596570</v>
+        <v>599795</v>
       </c>
       <c r="L686" s="6">
         <v>1110226</v>
       </c>
       <c r="M686" s="6">
-        <v>10221</v>
+        <v>14525</v>
       </c>
       <c r="N686" s="6">
-        <v>1120447</v>
+        <v>1124751</v>
       </c>
       <c r="O686" s="6">
-        <v>495882</v>
+        <v>496961</v>
       </c>
       <c r="P686" s="6">
         <v>26631</v>
@@ -56738,10 +56749,10 @@
         <v>177</v>
       </c>
       <c r="S686" s="6">
-        <v>523877</v>
+        <v>524956</v>
       </c>
       <c r="T686" s="6">
-        <v>538858</v>
+        <v>542083</v>
       </c>
       <c r="U686" s="6">
         <v>54295</v>
@@ -56753,10 +56764,10 @@
         <v>189</v>
       </c>
       <c r="X686" s="6">
-        <v>596570</v>
+        <v>599795</v>
       </c>
       <c r="Y686" s="6">
-        <v>1120447</v>
+        <v>1124751</v>
       </c>
       <c r="AA686" s="57"/>
     </row>
@@ -56780,34 +56791,34 @@
         <v>702695</v>
       </c>
       <c r="G687" s="6">
-        <v>6061</v>
+        <v>8369</v>
       </c>
       <c r="H687" s="6">
-        <v>708756</v>
+        <v>711064</v>
       </c>
       <c r="I687" s="6">
         <v>669414</v>
       </c>
       <c r="J687" s="6">
-        <v>3156</v>
+        <v>6344</v>
       </c>
       <c r="K687" s="6">
-        <v>672570</v>
+        <v>675758</v>
       </c>
       <c r="L687" s="6">
         <v>1372109</v>
       </c>
       <c r="M687" s="6">
-        <v>9217</v>
+        <v>14713</v>
       </c>
       <c r="N687" s="6">
-        <v>1381326</v>
+        <v>1386822</v>
       </c>
       <c r="O687" s="6">
-        <v>672299</v>
+        <v>674414</v>
       </c>
       <c r="P687" s="6">
-        <v>34602</v>
+        <v>34795</v>
       </c>
       <c r="Q687" s="6">
         <v>1810</v>
@@ -56816,10 +56827,10 @@
         <v>45</v>
       </c>
       <c r="S687" s="6">
-        <v>708756</v>
+        <v>711064</v>
       </c>
       <c r="T687" s="6">
-        <v>611287</v>
+        <v>614475</v>
       </c>
       <c r="U687" s="6">
         <v>57879</v>
@@ -56831,10 +56842,10 @@
         <v>138</v>
       </c>
       <c r="X687" s="6">
-        <v>672570</v>
+        <v>675758</v>
       </c>
       <c r="Y687" s="6">
-        <v>1381326</v>
+        <v>1386822</v>
       </c>
     </row>
     <row r="688" spans="1:27" x14ac:dyDescent="0.25">
@@ -56857,46 +56868,46 @@
         <v>456498</v>
       </c>
       <c r="G688" s="6">
-        <v>19214</v>
+        <v>41529</v>
       </c>
       <c r="H688" s="6">
-        <v>475712</v>
+        <v>498027</v>
       </c>
       <c r="I688" s="6">
         <v>390877</v>
       </c>
       <c r="J688" s="6">
-        <v>34640</v>
+        <v>74435</v>
       </c>
       <c r="K688" s="6">
-        <v>425517</v>
+        <v>465312</v>
       </c>
       <c r="L688" s="6">
         <v>847375</v>
       </c>
       <c r="M688" s="6">
-        <v>53854</v>
+        <v>115964</v>
       </c>
       <c r="N688" s="6">
-        <v>901229</v>
+        <v>963339</v>
       </c>
       <c r="O688" s="6">
-        <v>448500</v>
+        <v>470777</v>
       </c>
       <c r="P688" s="6">
-        <v>24519</v>
+        <v>24451</v>
       </c>
       <c r="Q688" s="6">
-        <v>2657</v>
+        <v>2763</v>
       </c>
       <c r="R688" s="6">
         <v>36</v>
       </c>
       <c r="S688" s="6">
-        <v>475712</v>
+        <v>498027</v>
       </c>
       <c r="T688" s="6">
-        <v>392966</v>
+        <v>432761</v>
       </c>
       <c r="U688" s="6">
         <v>31539</v>
@@ -56908,10 +56919,10 @@
         <v>188</v>
       </c>
       <c r="X688" s="6">
-        <v>425517</v>
+        <v>465312</v>
       </c>
       <c r="Y688" s="6">
-        <v>901229</v>
+        <v>963339</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -56934,31 +56945,31 @@
         <v>488226</v>
       </c>
       <c r="G689" s="6">
-        <v>884</v>
+        <v>5505</v>
       </c>
       <c r="H689" s="6">
-        <v>489110</v>
+        <v>493731</v>
       </c>
       <c r="I689" s="6">
         <v>379489</v>
       </c>
       <c r="J689" s="6">
-        <v>3001</v>
+        <v>3852</v>
       </c>
       <c r="K689" s="6">
-        <v>382490</v>
+        <v>383341</v>
       </c>
       <c r="L689" s="6">
         <v>867715</v>
       </c>
       <c r="M689" s="6">
-        <v>3885</v>
+        <v>9357</v>
       </c>
       <c r="N689" s="6">
-        <v>871600</v>
+        <v>877072</v>
       </c>
       <c r="O689" s="6">
-        <v>460578</v>
+        <v>465199</v>
       </c>
       <c r="P689" s="6">
         <v>25603</v>
@@ -56970,10 +56981,10 @@
         <v>45</v>
       </c>
       <c r="S689" s="6">
-        <v>489110</v>
+        <v>493731</v>
       </c>
       <c r="T689" s="6">
-        <v>350560</v>
+        <v>351411</v>
       </c>
       <c r="U689" s="6">
         <v>30516</v>
@@ -56985,10 +56996,10 @@
         <v>70</v>
       </c>
       <c r="X689" s="6">
-        <v>382490</v>
+        <v>383341</v>
       </c>
       <c r="Y689" s="6">
-        <v>871600</v>
+        <v>877072</v>
       </c>
     </row>
     <row r="690" spans="1:25" x14ac:dyDescent="0.25">
@@ -56998,7 +57009,7 @@
       <c r="B690" s="4">
         <v>19</v>
       </c>
-      <c r="C690" s="62" t="s">
+      <c r="C690" s="61" t="s">
         <v>731</v>
       </c>
       <c r="D690" s="6" t="s">
@@ -57011,34 +57022,34 @@
         <v>833175</v>
       </c>
       <c r="G690" s="6">
-        <v>0</v>
+        <v>3119</v>
       </c>
       <c r="H690" s="6">
-        <v>833175</v>
+        <v>836294</v>
       </c>
       <c r="I690" s="6">
         <v>556930</v>
       </c>
       <c r="J690" s="6">
-        <v>0</v>
+        <v>3233</v>
       </c>
       <c r="K690" s="6">
-        <v>556930</v>
+        <v>560163</v>
       </c>
       <c r="L690" s="6">
         <v>1390105</v>
       </c>
       <c r="M690" s="6">
-        <v>0</v>
+        <v>6352</v>
       </c>
       <c r="N690" s="6">
-        <v>1390105</v>
+        <v>1396457</v>
       </c>
       <c r="O690" s="6">
-        <v>785638</v>
+        <v>788687</v>
       </c>
       <c r="P690" s="6">
-        <v>42015</v>
+        <v>42085</v>
       </c>
       <c r="Q690" s="6">
         <v>5458</v>
@@ -57047,10 +57058,10 @@
         <v>64</v>
       </c>
       <c r="S690" s="6">
-        <v>833175</v>
+        <v>836294</v>
       </c>
       <c r="T690" s="6">
-        <v>496534</v>
+        <v>499767</v>
       </c>
       <c r="U690" s="6">
         <v>58245</v>
@@ -57062,10 +57073,10 @@
         <v>131</v>
       </c>
       <c r="X690" s="6">
-        <v>556930</v>
+        <v>560163</v>
       </c>
       <c r="Y690" s="6">
-        <v>1390105</v>
+        <v>1396457</v>
       </c>
     </row>
     <row r="691" spans="1:25" x14ac:dyDescent="0.25">
@@ -57075,33 +57086,75 @@
       <c r="B691" s="4">
         <v>20</v>
       </c>
-      <c r="C691" s="7"/>
+      <c r="C691" s="61" t="s">
+        <v>732</v>
+      </c>
       <c r="D691" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E691" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F691" s="6"/>
-      <c r="G691" s="6"/>
-      <c r="H691" s="6"/>
-      <c r="I691" s="6"/>
-      <c r="J691" s="6"/>
-      <c r="K691" s="6"/>
-      <c r="L691" s="6"/>
-      <c r="M691" s="6"/>
-      <c r="N691" s="6"/>
-      <c r="O691" s="6"/>
-      <c r="P691" s="6"/>
-      <c r="Q691" s="6"/>
-      <c r="R691" s="6"/>
-      <c r="S691" s="6"/>
-      <c r="T691" s="6"/>
-      <c r="U691" s="6"/>
-      <c r="V691" s="6"/>
-      <c r="W691" s="6"/>
-      <c r="X691" s="6"/>
-      <c r="Y691" s="6"/>
+      <c r="F691" s="6">
+        <v>915075</v>
+      </c>
+      <c r="G691" s="6">
+        <v>10532</v>
+      </c>
+      <c r="H691" s="6">
+        <v>925607</v>
+      </c>
+      <c r="I691" s="6">
+        <v>550540</v>
+      </c>
+      <c r="J691" s="6">
+        <v>2584</v>
+      </c>
+      <c r="K691" s="6">
+        <v>553124</v>
+      </c>
+      <c r="L691" s="6">
+        <v>1465615</v>
+      </c>
+      <c r="M691" s="6">
+        <v>13116</v>
+      </c>
+      <c r="N691" s="6">
+        <v>1478731</v>
+      </c>
+      <c r="O691" s="6">
+        <v>870358</v>
+      </c>
+      <c r="P691" s="6">
+        <v>51271</v>
+      </c>
+      <c r="Q691" s="6">
+        <v>3900</v>
+      </c>
+      <c r="R691" s="6">
+        <v>78</v>
+      </c>
+      <c r="S691" s="6">
+        <v>925607</v>
+      </c>
+      <c r="T691" s="6">
+        <v>496750</v>
+      </c>
+      <c r="U691" s="6">
+        <v>52748</v>
+      </c>
+      <c r="V691" s="6">
+        <v>3488</v>
+      </c>
+      <c r="W691" s="6">
+        <v>138</v>
+      </c>
+      <c r="X691" s="6">
+        <v>553124</v>
+      </c>
+      <c r="Y691" s="6">
+        <v>1478731</v>
+      </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A692" s="7">
@@ -57110,33 +57163,75 @@
       <c r="B692" s="4">
         <v>21</v>
       </c>
-      <c r="C692" s="7"/>
+      <c r="C692" s="62" t="s">
+        <v>733</v>
+      </c>
       <c r="D692" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E692" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F692" s="6"/>
-      <c r="G692" s="6"/>
-      <c r="H692" s="6"/>
-      <c r="I692" s="6"/>
-      <c r="J692" s="6"/>
-      <c r="K692" s="6"/>
-      <c r="L692" s="6"/>
-      <c r="M692" s="6"/>
-      <c r="N692" s="6"/>
-      <c r="O692" s="6"/>
-      <c r="P692" s="6"/>
-      <c r="Q692" s="6"/>
-      <c r="R692" s="6"/>
-      <c r="S692" s="6"/>
-      <c r="T692" s="6"/>
-      <c r="U692" s="6"/>
-      <c r="V692" s="6"/>
-      <c r="W692" s="6"/>
-      <c r="X692" s="6"/>
-      <c r="Y692" s="6"/>
+      <c r="F692" s="6">
+        <v>937765</v>
+      </c>
+      <c r="G692" s="6">
+        <v>0</v>
+      </c>
+      <c r="H692" s="6">
+        <v>937765</v>
+      </c>
+      <c r="I692" s="6">
+        <v>445313</v>
+      </c>
+      <c r="J692" s="6">
+        <v>0</v>
+      </c>
+      <c r="K692" s="6">
+        <v>445313</v>
+      </c>
+      <c r="L692" s="6">
+        <v>1383078</v>
+      </c>
+      <c r="M692" s="6">
+        <v>0</v>
+      </c>
+      <c r="N692" s="6">
+        <v>1383078</v>
+      </c>
+      <c r="O692" s="6">
+        <v>873620</v>
+      </c>
+      <c r="P692" s="6">
+        <v>61445</v>
+      </c>
+      <c r="Q692" s="6">
+        <v>2678</v>
+      </c>
+      <c r="R692" s="6">
+        <v>22</v>
+      </c>
+      <c r="S692" s="6">
+        <v>937765</v>
+      </c>
+      <c r="T692" s="6">
+        <v>390836</v>
+      </c>
+      <c r="U692" s="6">
+        <v>51710</v>
+      </c>
+      <c r="V692" s="6">
+        <v>2697</v>
+      </c>
+      <c r="W692" s="6">
+        <v>70</v>
+      </c>
+      <c r="X692" s="6">
+        <v>445313</v>
+      </c>
+      <c r="Y692" s="6">
+        <v>1383078</v>
+      </c>
     </row>
     <row r="693" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A693" s="7">
@@ -58493,26 +58588,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -58739,26 +58814,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
-    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -58775,4 +58851,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
+    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Daily project backup 2026-08-05
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E92842-B669-42CD-A72F-D1D679DE64B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F8E02D9-0156-4B05-9EA3-D4D1EA1566AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28980" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2186" uniqueCount="734">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="735">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2238,6 +2238,9 @@
   </si>
   <si>
     <t>18/07 - 24/07/2026</t>
+  </si>
+  <si>
+    <t>25/07 - 31/07/2026</t>
   </si>
 </sst>
 </file>
@@ -2791,15 +2794,15 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3173,11 +3176,11 @@
         <v>76</v>
       </c>
       <c r="AC1" s="45"/>
-      <c r="AD1" s="58" t="s">
+      <c r="AD1" s="61" t="s">
         <v>723</v>
       </c>
-      <c r="AE1" s="58"/>
-      <c r="AF1" s="59"/>
+      <c r="AE1" s="61"/>
+      <c r="AF1" s="62"/>
     </row>
     <row r="2" spans="1:32" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31">
@@ -56231,7 +56234,7 @@
       <c r="B680" s="18">
         <v>9</v>
       </c>
-      <c r="C680" s="60" t="s">
+      <c r="C680" s="58" t="s">
         <v>78</v>
       </c>
       <c r="D680" s="15" t="s">
@@ -56310,7 +56313,7 @@
       <c r="B681" s="4">
         <v>10</v>
       </c>
-      <c r="C681" s="61" t="s">
+      <c r="C681" s="59" t="s">
         <v>79</v>
       </c>
       <c r="D681" s="6" t="s">
@@ -56388,7 +56391,7 @@
       <c r="B682" s="4">
         <v>11</v>
       </c>
-      <c r="C682" s="61" t="s">
+      <c r="C682" s="59" t="s">
         <v>80</v>
       </c>
       <c r="D682" s="6" t="s">
@@ -56466,7 +56469,7 @@
       <c r="B683" s="4">
         <v>12</v>
       </c>
-      <c r="C683" s="61" t="s">
+      <c r="C683" s="59" t="s">
         <v>81</v>
       </c>
       <c r="D683" s="6" t="s">
@@ -56488,19 +56491,19 @@
         <v>285962</v>
       </c>
       <c r="J683" s="10">
-        <v>2824</v>
+        <v>2860</v>
       </c>
       <c r="K683" s="10">
-        <v>288786</v>
+        <v>288822</v>
       </c>
       <c r="L683" s="10">
         <v>406821</v>
       </c>
       <c r="M683" s="10">
-        <v>2631</v>
+        <v>2667</v>
       </c>
       <c r="N683" s="10">
-        <v>409452</v>
+        <v>409488</v>
       </c>
       <c r="O683" s="10">
         <v>115619</v>
@@ -56518,7 +56521,7 @@
         <v>120666</v>
       </c>
       <c r="T683" s="10">
-        <v>277428</v>
+        <v>277464</v>
       </c>
       <c r="U683" s="10">
         <v>10777</v>
@@ -56530,10 +56533,10 @@
         <v>2</v>
       </c>
       <c r="X683" s="10">
-        <v>288786</v>
+        <v>288822</v>
       </c>
       <c r="Y683" s="10">
-        <v>409452</v>
+        <v>409488</v>
       </c>
       <c r="AA683" s="57"/>
     </row>
@@ -56544,7 +56547,7 @@
       <c r="B684" s="4">
         <v>13</v>
       </c>
-      <c r="C684" s="61" t="s">
+      <c r="C684" s="59" t="s">
         <v>82</v>
       </c>
       <c r="D684" s="6" t="s">
@@ -56622,7 +56625,7 @@
       <c r="B685" s="4">
         <v>14</v>
       </c>
-      <c r="C685" s="61" t="s">
+      <c r="C685" s="59" t="s">
         <v>83</v>
       </c>
       <c r="D685" s="6" t="s">
@@ -56700,7 +56703,7 @@
       <c r="B686" s="4">
         <v>15</v>
       </c>
-      <c r="C686" s="61" t="s">
+      <c r="C686" s="59" t="s">
         <v>727</v>
       </c>
       <c r="D686" s="6" t="s">
@@ -56778,7 +56781,7 @@
       <c r="B687" s="4">
         <v>16</v>
       </c>
-      <c r="C687" s="61" t="s">
+      <c r="C687" s="59" t="s">
         <v>728</v>
       </c>
       <c r="D687" s="6" t="s">
@@ -56855,7 +56858,7 @@
       <c r="B688" s="4">
         <v>17</v>
       </c>
-      <c r="C688" s="61" t="s">
+      <c r="C688" s="59" t="s">
         <v>729</v>
       </c>
       <c r="D688" s="6" t="s">
@@ -56868,10 +56871,10 @@
         <v>456498</v>
       </c>
       <c r="G688" s="6">
-        <v>41529</v>
+        <v>42779</v>
       </c>
       <c r="H688" s="6">
-        <v>498027</v>
+        <v>499277</v>
       </c>
       <c r="I688" s="6">
         <v>390877</v>
@@ -56886,13 +56889,13 @@
         <v>847375</v>
       </c>
       <c r="M688" s="6">
-        <v>115964</v>
+        <v>117214</v>
       </c>
       <c r="N688" s="6">
-        <v>963339</v>
+        <v>964589</v>
       </c>
       <c r="O688" s="6">
-        <v>470777</v>
+        <v>472027</v>
       </c>
       <c r="P688" s="6">
         <v>24451</v>
@@ -56904,7 +56907,7 @@
         <v>36</v>
       </c>
       <c r="S688" s="6">
-        <v>498027</v>
+        <v>499277</v>
       </c>
       <c r="T688" s="6">
         <v>432761</v>
@@ -56922,7 +56925,7 @@
         <v>465312</v>
       </c>
       <c r="Y688" s="6">
-        <v>963339</v>
+        <v>964589</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -56932,7 +56935,7 @@
       <c r="B689" s="4">
         <v>18</v>
       </c>
-      <c r="C689" s="61" t="s">
+      <c r="C689" s="59" t="s">
         <v>730</v>
       </c>
       <c r="D689" s="6" t="s">
@@ -57009,7 +57012,7 @@
       <c r="B690" s="4">
         <v>19</v>
       </c>
-      <c r="C690" s="61" t="s">
+      <c r="C690" s="59" t="s">
         <v>731</v>
       </c>
       <c r="D690" s="6" t="s">
@@ -57022,19 +57025,19 @@
         <v>833175</v>
       </c>
       <c r="G690" s="6">
-        <v>3119</v>
+        <v>3156</v>
       </c>
       <c r="H690" s="6">
-        <v>836294</v>
+        <v>836331</v>
       </c>
       <c r="I690" s="6">
         <v>556930</v>
       </c>
       <c r="J690" s="6">
-        <v>3233</v>
+        <v>3196</v>
       </c>
       <c r="K690" s="6">
-        <v>560163</v>
+        <v>560126</v>
       </c>
       <c r="L690" s="6">
         <v>1390105</v>
@@ -57046,7 +57049,7 @@
         <v>1396457</v>
       </c>
       <c r="O690" s="6">
-        <v>788687</v>
+        <v>788724</v>
       </c>
       <c r="P690" s="6">
         <v>42085</v>
@@ -57058,10 +57061,10 @@
         <v>64</v>
       </c>
       <c r="S690" s="6">
-        <v>836294</v>
+        <v>836331</v>
       </c>
       <c r="T690" s="6">
-        <v>499767</v>
+        <v>499730</v>
       </c>
       <c r="U690" s="6">
         <v>58245</v>
@@ -57073,7 +57076,7 @@
         <v>131</v>
       </c>
       <c r="X690" s="6">
-        <v>560163</v>
+        <v>560126</v>
       </c>
       <c r="Y690" s="6">
         <v>1396457</v>
@@ -57086,7 +57089,7 @@
       <c r="B691" s="4">
         <v>20</v>
       </c>
-      <c r="C691" s="61" t="s">
+      <c r="C691" s="59" t="s">
         <v>732</v>
       </c>
       <c r="D691" s="6" t="s">
@@ -57108,19 +57111,19 @@
         <v>550540</v>
       </c>
       <c r="J691" s="6">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="K691" s="6">
-        <v>553124</v>
+        <v>553125</v>
       </c>
       <c r="L691" s="6">
         <v>1465615</v>
       </c>
       <c r="M691" s="6">
-        <v>13116</v>
+        <v>13117</v>
       </c>
       <c r="N691" s="6">
-        <v>1478731</v>
+        <v>1478732</v>
       </c>
       <c r="O691" s="6">
         <v>870358</v>
@@ -57138,7 +57141,7 @@
         <v>925607</v>
       </c>
       <c r="T691" s="6">
-        <v>496750</v>
+        <v>496751</v>
       </c>
       <c r="U691" s="6">
         <v>52748</v>
@@ -57150,10 +57153,10 @@
         <v>138</v>
       </c>
       <c r="X691" s="6">
-        <v>553124</v>
+        <v>553125</v>
       </c>
       <c r="Y691" s="6">
-        <v>1478731</v>
+        <v>1478732</v>
       </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
@@ -57163,7 +57166,7 @@
       <c r="B692" s="4">
         <v>21</v>
       </c>
-      <c r="C692" s="62" t="s">
+      <c r="C692" s="59" t="s">
         <v>733</v>
       </c>
       <c r="D692" s="6" t="s">
@@ -57176,31 +57179,31 @@
         <v>937765</v>
       </c>
       <c r="G692" s="6">
-        <v>0</v>
+        <v>2904</v>
       </c>
       <c r="H692" s="6">
-        <v>937765</v>
+        <v>940669</v>
       </c>
       <c r="I692" s="6">
         <v>445313</v>
       </c>
       <c r="J692" s="6">
-        <v>0</v>
+        <v>12201</v>
       </c>
       <c r="K692" s="6">
-        <v>445313</v>
+        <v>457514</v>
       </c>
       <c r="L692" s="6">
         <v>1383078</v>
       </c>
       <c r="M692" s="6">
-        <v>0</v>
+        <v>15105</v>
       </c>
       <c r="N692" s="6">
-        <v>1383078</v>
+        <v>1398183</v>
       </c>
       <c r="O692" s="6">
-        <v>873620</v>
+        <v>876524</v>
       </c>
       <c r="P692" s="6">
         <v>61445</v>
@@ -57212,13 +57215,13 @@
         <v>22</v>
       </c>
       <c r="S692" s="6">
-        <v>937765</v>
+        <v>940669</v>
       </c>
       <c r="T692" s="6">
-        <v>390836</v>
+        <v>402584</v>
       </c>
       <c r="U692" s="6">
-        <v>51710</v>
+        <v>52163</v>
       </c>
       <c r="V692" s="6">
         <v>2697</v>
@@ -57227,10 +57230,10 @@
         <v>70</v>
       </c>
       <c r="X692" s="6">
-        <v>445313</v>
+        <v>457514</v>
       </c>
       <c r="Y692" s="6">
-        <v>1383078</v>
+        <v>1398183</v>
       </c>
     </row>
     <row r="693" spans="1:25" x14ac:dyDescent="0.25">
@@ -57240,33 +57243,75 @@
       <c r="B693" s="4">
         <v>22</v>
       </c>
-      <c r="C693" s="7"/>
+      <c r="C693" s="60" t="s">
+        <v>734</v>
+      </c>
       <c r="D693" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E693" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F693" s="6"/>
-      <c r="G693" s="6"/>
-      <c r="H693" s="6"/>
-      <c r="I693" s="6"/>
-      <c r="J693" s="6"/>
-      <c r="K693" s="6"/>
-      <c r="L693" s="6"/>
-      <c r="M693" s="6"/>
-      <c r="N693" s="6"/>
-      <c r="O693" s="6"/>
-      <c r="P693" s="6"/>
-      <c r="Q693" s="6"/>
-      <c r="R693" s="6"/>
-      <c r="S693" s="6"/>
-      <c r="T693" s="6"/>
-      <c r="U693" s="6"/>
-      <c r="V693" s="6"/>
-      <c r="W693" s="6"/>
-      <c r="X693" s="6"/>
-      <c r="Y693" s="6"/>
+      <c r="F693" s="6">
+        <v>800679</v>
+      </c>
+      <c r="G693" s="6">
+        <v>0</v>
+      </c>
+      <c r="H693" s="6">
+        <v>800679</v>
+      </c>
+      <c r="I693" s="6">
+        <v>343793</v>
+      </c>
+      <c r="J693" s="6">
+        <v>0</v>
+      </c>
+      <c r="K693" s="6">
+        <v>343793</v>
+      </c>
+      <c r="L693" s="6">
+        <v>1144472</v>
+      </c>
+      <c r="M693" s="6">
+        <v>0</v>
+      </c>
+      <c r="N693" s="6">
+        <v>1144472</v>
+      </c>
+      <c r="O693" s="6">
+        <v>734845</v>
+      </c>
+      <c r="P693" s="6">
+        <v>62200</v>
+      </c>
+      <c r="Q693" s="6">
+        <v>3628</v>
+      </c>
+      <c r="R693" s="6">
+        <v>6</v>
+      </c>
+      <c r="S693" s="6">
+        <v>800679</v>
+      </c>
+      <c r="T693" s="6">
+        <v>302490</v>
+      </c>
+      <c r="U693" s="6">
+        <v>40392</v>
+      </c>
+      <c r="V693" s="6">
+        <v>887</v>
+      </c>
+      <c r="W693" s="6">
+        <v>24</v>
+      </c>
+      <c r="X693" s="6">
+        <v>343793</v>
+      </c>
+      <c r="Y693" s="6">
+        <v>1144472</v>
+      </c>
     </row>
     <row r="694" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A694" s="7">
@@ -58588,6 +58633,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -58814,15 +58868,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -58835,6 +58880,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -58853,14 +58906,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update AGR prices and commodity deliveries
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F8E02D9-0156-4B05-9EA3-D4D1EA1566AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC5FA266-2280-4072-ABC8-ECD8D143F726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28980" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-16200" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="735">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2188" uniqueCount="736">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2241,6 +2241,9 @@
   </si>
   <si>
     <t>25/07 - 31/07/2026</t>
+  </si>
+  <si>
+    <t>01/08 - 07/08/2026</t>
   </si>
 </sst>
 </file>
@@ -56569,19 +56572,19 @@
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>33866</v>
+        <v>34173</v>
       </c>
       <c r="K684" s="10">
-        <v>446725</v>
+        <v>447032</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>45141</v>
+        <v>45448</v>
       </c>
       <c r="N684" s="10">
-        <v>659415</v>
+        <v>659722</v>
       </c>
       <c r="O684" s="10">
         <v>203773</v>
@@ -56599,7 +56602,7 @@
         <v>212690</v>
       </c>
       <c r="T684" s="10">
-        <v>422975</v>
+        <v>423282</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56611,10 +56614,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>446725</v>
+        <v>447032</v>
       </c>
       <c r="Y684" s="10">
-        <v>659415</v>
+        <v>659722</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56871,31 +56874,31 @@
         <v>456498</v>
       </c>
       <c r="G688" s="6">
-        <v>42779</v>
+        <v>43178</v>
       </c>
       <c r="H688" s="6">
-        <v>499277</v>
+        <v>499676</v>
       </c>
       <c r="I688" s="6">
         <v>390877</v>
       </c>
       <c r="J688" s="6">
-        <v>74435</v>
+        <v>74793</v>
       </c>
       <c r="K688" s="6">
-        <v>465312</v>
+        <v>465670</v>
       </c>
       <c r="L688" s="6">
         <v>847375</v>
       </c>
       <c r="M688" s="6">
-        <v>117214</v>
+        <v>117971</v>
       </c>
       <c r="N688" s="6">
-        <v>964589</v>
+        <v>965346</v>
       </c>
       <c r="O688" s="6">
-        <v>472027</v>
+        <v>472426</v>
       </c>
       <c r="P688" s="6">
         <v>24451</v>
@@ -56907,10 +56910,10 @@
         <v>36</v>
       </c>
       <c r="S688" s="6">
-        <v>499277</v>
+        <v>499676</v>
       </c>
       <c r="T688" s="6">
-        <v>432761</v>
+        <v>433119</v>
       </c>
       <c r="U688" s="6">
         <v>31539</v>
@@ -56922,10 +56925,10 @@
         <v>188</v>
       </c>
       <c r="X688" s="6">
-        <v>465312</v>
+        <v>465670</v>
       </c>
       <c r="Y688" s="6">
-        <v>964589</v>
+        <v>965346</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -57025,31 +57028,31 @@
         <v>833175</v>
       </c>
       <c r="G690" s="6">
-        <v>3156</v>
+        <v>3331</v>
       </c>
       <c r="H690" s="6">
-        <v>836331</v>
+        <v>836506</v>
       </c>
       <c r="I690" s="6">
         <v>556930</v>
       </c>
       <c r="J690" s="6">
-        <v>3196</v>
+        <v>3247</v>
       </c>
       <c r="K690" s="6">
-        <v>560126</v>
+        <v>560177</v>
       </c>
       <c r="L690" s="6">
         <v>1390105</v>
       </c>
       <c r="M690" s="6">
-        <v>6352</v>
+        <v>6578</v>
       </c>
       <c r="N690" s="6">
-        <v>1396457</v>
+        <v>1396683</v>
       </c>
       <c r="O690" s="6">
-        <v>788724</v>
+        <v>788899</v>
       </c>
       <c r="P690" s="6">
         <v>42085</v>
@@ -57061,10 +57064,10 @@
         <v>64</v>
       </c>
       <c r="S690" s="6">
-        <v>836331</v>
+        <v>836506</v>
       </c>
       <c r="T690" s="6">
-        <v>499730</v>
+        <v>499781</v>
       </c>
       <c r="U690" s="6">
         <v>58245</v>
@@ -57076,10 +57079,10 @@
         <v>131</v>
       </c>
       <c r="X690" s="6">
-        <v>560126</v>
+        <v>560177</v>
       </c>
       <c r="Y690" s="6">
-        <v>1396457</v>
+        <v>1396683</v>
       </c>
     </row>
     <row r="691" spans="1:25" x14ac:dyDescent="0.25">
@@ -57102,31 +57105,31 @@
         <v>915075</v>
       </c>
       <c r="G691" s="6">
-        <v>10532</v>
+        <v>10849</v>
       </c>
       <c r="H691" s="6">
-        <v>925607</v>
+        <v>925924</v>
       </c>
       <c r="I691" s="6">
         <v>550540</v>
       </c>
       <c r="J691" s="6">
-        <v>2585</v>
+        <v>3446</v>
       </c>
       <c r="K691" s="6">
-        <v>553125</v>
+        <v>553986</v>
       </c>
       <c r="L691" s="6">
         <v>1465615</v>
       </c>
       <c r="M691" s="6">
-        <v>13117</v>
+        <v>14295</v>
       </c>
       <c r="N691" s="6">
-        <v>1478732</v>
+        <v>1479910</v>
       </c>
       <c r="O691" s="6">
-        <v>870358</v>
+        <v>870675</v>
       </c>
       <c r="P691" s="6">
         <v>51271</v>
@@ -57138,10 +57141,10 @@
         <v>78</v>
       </c>
       <c r="S691" s="6">
-        <v>925607</v>
+        <v>925924</v>
       </c>
       <c r="T691" s="6">
-        <v>496751</v>
+        <v>497612</v>
       </c>
       <c r="U691" s="6">
         <v>52748</v>
@@ -57153,10 +57156,10 @@
         <v>138</v>
       </c>
       <c r="X691" s="6">
-        <v>553125</v>
+        <v>553986</v>
       </c>
       <c r="Y691" s="6">
-        <v>1478732</v>
+        <v>1479910</v>
       </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
@@ -57179,31 +57182,31 @@
         <v>937765</v>
       </c>
       <c r="G692" s="6">
-        <v>2904</v>
+        <v>2917</v>
       </c>
       <c r="H692" s="6">
-        <v>940669</v>
+        <v>940682</v>
       </c>
       <c r="I692" s="6">
         <v>445313</v>
       </c>
       <c r="J692" s="6">
-        <v>12201</v>
+        <v>12763</v>
       </c>
       <c r="K692" s="6">
-        <v>457514</v>
+        <v>458076</v>
       </c>
       <c r="L692" s="6">
         <v>1383078</v>
       </c>
       <c r="M692" s="6">
-        <v>15105</v>
+        <v>15680</v>
       </c>
       <c r="N692" s="6">
-        <v>1398183</v>
+        <v>1398758</v>
       </c>
       <c r="O692" s="6">
-        <v>876524</v>
+        <v>876537</v>
       </c>
       <c r="P692" s="6">
         <v>61445</v>
@@ -57215,10 +57218,10 @@
         <v>22</v>
       </c>
       <c r="S692" s="6">
-        <v>940669</v>
+        <v>940682</v>
       </c>
       <c r="T692" s="6">
-        <v>402584</v>
+        <v>403146</v>
       </c>
       <c r="U692" s="6">
         <v>52163</v>
@@ -57230,10 +57233,10 @@
         <v>70</v>
       </c>
       <c r="X692" s="6">
-        <v>457514</v>
+        <v>458076</v>
       </c>
       <c r="Y692" s="6">
-        <v>1398183</v>
+        <v>1398758</v>
       </c>
     </row>
     <row r="693" spans="1:25" x14ac:dyDescent="0.25">
@@ -57243,7 +57246,7 @@
       <c r="B693" s="4">
         <v>22</v>
       </c>
-      <c r="C693" s="60" t="s">
+      <c r="C693" s="59" t="s">
         <v>734</v>
       </c>
       <c r="D693" s="6" t="s">
@@ -57256,34 +57259,34 @@
         <v>800679</v>
       </c>
       <c r="G693" s="6">
-        <v>0</v>
+        <v>16871</v>
       </c>
       <c r="H693" s="6">
-        <v>800679</v>
+        <v>817550</v>
       </c>
       <c r="I693" s="6">
         <v>343793</v>
       </c>
       <c r="J693" s="6">
-        <v>0</v>
+        <v>33956</v>
       </c>
       <c r="K693" s="6">
-        <v>343793</v>
+        <v>377749</v>
       </c>
       <c r="L693" s="6">
         <v>1144472</v>
       </c>
       <c r="M693" s="6">
-        <v>0</v>
+        <v>50827</v>
       </c>
       <c r="N693" s="6">
-        <v>1144472</v>
+        <v>1195299</v>
       </c>
       <c r="O693" s="6">
-        <v>734845</v>
+        <v>751641</v>
       </c>
       <c r="P693" s="6">
-        <v>62200</v>
+        <v>62275</v>
       </c>
       <c r="Q693" s="6">
         <v>3628</v>
@@ -57292,13 +57295,13 @@
         <v>6</v>
       </c>
       <c r="S693" s="6">
-        <v>800679</v>
+        <v>817550</v>
       </c>
       <c r="T693" s="6">
-        <v>302490</v>
+        <v>336374</v>
       </c>
       <c r="U693" s="6">
-        <v>40392</v>
+        <v>40464</v>
       </c>
       <c r="V693" s="6">
         <v>887</v>
@@ -57307,10 +57310,10 @@
         <v>24</v>
       </c>
       <c r="X693" s="6">
-        <v>343793</v>
+        <v>377749</v>
       </c>
       <c r="Y693" s="6">
-        <v>1144472</v>
+        <v>1195299</v>
       </c>
     </row>
     <row r="694" spans="1:25" x14ac:dyDescent="0.25">
@@ -57320,33 +57323,75 @@
       <c r="B694" s="4">
         <v>23</v>
       </c>
-      <c r="C694" s="7"/>
+      <c r="C694" s="60" t="s">
+        <v>735</v>
+      </c>
       <c r="D694" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E694" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F694" s="6"/>
-      <c r="G694" s="6"/>
-      <c r="H694" s="6"/>
-      <c r="I694" s="6"/>
-      <c r="J694" s="6"/>
-      <c r="K694" s="6"/>
-      <c r="L694" s="6"/>
-      <c r="M694" s="6"/>
-      <c r="N694" s="6"/>
-      <c r="O694" s="6"/>
-      <c r="P694" s="6"/>
-      <c r="Q694" s="6"/>
-      <c r="R694" s="6"/>
-      <c r="S694" s="6"/>
-      <c r="T694" s="6"/>
-      <c r="U694" s="6"/>
-      <c r="V694" s="6"/>
-      <c r="W694" s="6"/>
-      <c r="X694" s="6"/>
-      <c r="Y694" s="6"/>
+      <c r="F694" s="6">
+        <v>637394</v>
+      </c>
+      <c r="G694" s="6">
+        <v>0</v>
+      </c>
+      <c r="H694" s="6">
+        <v>637394</v>
+      </c>
+      <c r="I694" s="6">
+        <v>257890</v>
+      </c>
+      <c r="J694" s="6">
+        <v>0</v>
+      </c>
+      <c r="K694" s="6">
+        <v>257890</v>
+      </c>
+      <c r="L694" s="6">
+        <v>895284</v>
+      </c>
+      <c r="M694" s="6">
+        <v>0</v>
+      </c>
+      <c r="N694" s="6">
+        <v>895284</v>
+      </c>
+      <c r="O694" s="6">
+        <v>572666</v>
+      </c>
+      <c r="P694" s="6">
+        <v>61784</v>
+      </c>
+      <c r="Q694" s="6">
+        <v>2918</v>
+      </c>
+      <c r="R694" s="6">
+        <v>26</v>
+      </c>
+      <c r="S694" s="6">
+        <v>637394</v>
+      </c>
+      <c r="T694" s="6">
+        <v>228745</v>
+      </c>
+      <c r="U694" s="6">
+        <v>28327</v>
+      </c>
+      <c r="V694" s="6">
+        <v>783</v>
+      </c>
+      <c r="W694" s="6">
+        <v>35</v>
+      </c>
+      <c r="X694" s="6">
+        <v>257890</v>
+      </c>
+      <c r="Y694" s="6">
+        <v>895284</v>
+      </c>
     </row>
     <row r="695" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A695" s="7">
@@ -58633,15 +58678,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -58868,6 +58904,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -58880,14 +58925,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -58906,6 +58943,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update White Maize CEC crop estimate
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC5FA266-2280-4072-ABC8-ECD8D143F726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F51FCBB8-B163-4014-914B-1F848D3D8538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-16200" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4525,14 +4525,14 @@
         <v>77</v>
       </c>
       <c r="AD16" s="51">
-        <v>9282690</v>
+        <v>9390790</v>
       </c>
       <c r="AE16" s="51">
         <v>7971850</v>
       </c>
       <c r="AF16" s="53">
         <f>AE16+AD16</f>
-        <v>17254540</v>
+        <v>17362640</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
@@ -58905,15 +58905,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
@@ -58922,6 +58913,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -58944,14 +58944,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -58960,4 +58952,12 @@
     <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update AGR and deliveries data
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F51FCBB8-B163-4014-914B-1F848D3D8538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{538A65DB-1B84-44A0-B0D1-8097CA8570A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-16200" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16335" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2188" uniqueCount="736">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2189" uniqueCount="737">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2244,6 +2244,9 @@
   </si>
   <si>
     <t>01/08 - 07/08/2026</t>
+  </si>
+  <si>
+    <t>08/08 - 14/08/2026</t>
   </si>
 </sst>
 </file>
@@ -56572,19 +56575,19 @@
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>34173</v>
+        <v>34205</v>
       </c>
       <c r="K684" s="10">
-        <v>447032</v>
+        <v>447064</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>45448</v>
+        <v>45480</v>
       </c>
       <c r="N684" s="10">
-        <v>659722</v>
+        <v>659754</v>
       </c>
       <c r="O684" s="10">
         <v>203773</v>
@@ -56602,7 +56605,7 @@
         <v>212690</v>
       </c>
       <c r="T684" s="10">
-        <v>423282</v>
+        <v>423314</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56614,10 +56617,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>447032</v>
+        <v>447064</v>
       </c>
       <c r="Y684" s="10">
-        <v>659722</v>
+        <v>659754</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56874,10 +56877,10 @@
         <v>456498</v>
       </c>
       <c r="G688" s="6">
-        <v>43178</v>
+        <v>46724</v>
       </c>
       <c r="H688" s="6">
-        <v>499676</v>
+        <v>503222</v>
       </c>
       <c r="I688" s="6">
         <v>390877</v>
@@ -56892,13 +56895,13 @@
         <v>847375</v>
       </c>
       <c r="M688" s="6">
-        <v>117971</v>
+        <v>121517</v>
       </c>
       <c r="N688" s="6">
-        <v>965346</v>
+        <v>968892</v>
       </c>
       <c r="O688" s="6">
-        <v>472426</v>
+        <v>475972</v>
       </c>
       <c r="P688" s="6">
         <v>24451</v>
@@ -56910,7 +56913,7 @@
         <v>36</v>
       </c>
       <c r="S688" s="6">
-        <v>499676</v>
+        <v>503222</v>
       </c>
       <c r="T688" s="6">
         <v>433119</v>
@@ -56928,7 +56931,7 @@
         <v>465670</v>
       </c>
       <c r="Y688" s="6">
-        <v>965346</v>
+        <v>968892</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -56951,31 +56954,31 @@
         <v>488226</v>
       </c>
       <c r="G689" s="6">
-        <v>5505</v>
+        <v>6304</v>
       </c>
       <c r="H689" s="6">
-        <v>493731</v>
+        <v>494530</v>
       </c>
       <c r="I689" s="6">
         <v>379489</v>
       </c>
       <c r="J689" s="6">
-        <v>3852</v>
+        <v>13355</v>
       </c>
       <c r="K689" s="6">
-        <v>383341</v>
+        <v>392844</v>
       </c>
       <c r="L689" s="6">
         <v>867715</v>
       </c>
       <c r="M689" s="6">
-        <v>9357</v>
+        <v>19659</v>
       </c>
       <c r="N689" s="6">
-        <v>877072</v>
+        <v>887374</v>
       </c>
       <c r="O689" s="6">
-        <v>465199</v>
+        <v>465998</v>
       </c>
       <c r="P689" s="6">
         <v>25603</v>
@@ -56987,25 +56990,25 @@
         <v>45</v>
       </c>
       <c r="S689" s="6">
-        <v>493731</v>
+        <v>494530</v>
       </c>
       <c r="T689" s="6">
-        <v>351411</v>
+        <v>358168</v>
       </c>
       <c r="U689" s="6">
-        <v>30516</v>
+        <v>33163</v>
       </c>
       <c r="V689" s="6">
-        <v>1344</v>
+        <v>1443</v>
       </c>
       <c r="W689" s="6">
         <v>70</v>
       </c>
       <c r="X689" s="6">
-        <v>383341</v>
+        <v>392844</v>
       </c>
       <c r="Y689" s="6">
-        <v>877072</v>
+        <v>887374</v>
       </c>
     </row>
     <row r="690" spans="1:25" x14ac:dyDescent="0.25">
@@ -57028,31 +57031,31 @@
         <v>833175</v>
       </c>
       <c r="G690" s="6">
-        <v>3331</v>
+        <v>9035</v>
       </c>
       <c r="H690" s="6">
-        <v>836506</v>
+        <v>842210</v>
       </c>
       <c r="I690" s="6">
         <v>556930</v>
       </c>
       <c r="J690" s="6">
-        <v>3247</v>
+        <v>6465</v>
       </c>
       <c r="K690" s="6">
-        <v>560177</v>
+        <v>563395</v>
       </c>
       <c r="L690" s="6">
         <v>1390105</v>
       </c>
       <c r="M690" s="6">
-        <v>6578</v>
+        <v>15500</v>
       </c>
       <c r="N690" s="6">
-        <v>1396683</v>
+        <v>1405605</v>
       </c>
       <c r="O690" s="6">
-        <v>788899</v>
+        <v>794603</v>
       </c>
       <c r="P690" s="6">
         <v>42085</v>
@@ -57064,25 +57067,25 @@
         <v>64</v>
       </c>
       <c r="S690" s="6">
-        <v>836506</v>
+        <v>842210</v>
       </c>
       <c r="T690" s="6">
-        <v>499781</v>
+        <v>502494</v>
       </c>
       <c r="U690" s="6">
-        <v>58245</v>
+        <v>58757</v>
       </c>
       <c r="V690" s="6">
-        <v>2020</v>
+        <v>2013</v>
       </c>
       <c r="W690" s="6">
         <v>131</v>
       </c>
       <c r="X690" s="6">
-        <v>560177</v>
+        <v>563395</v>
       </c>
       <c r="Y690" s="6">
-        <v>1396683</v>
+        <v>1405605</v>
       </c>
     </row>
     <row r="691" spans="1:25" x14ac:dyDescent="0.25">
@@ -57105,31 +57108,31 @@
         <v>915075</v>
       </c>
       <c r="G691" s="6">
-        <v>10849</v>
+        <v>37654</v>
       </c>
       <c r="H691" s="6">
-        <v>925924</v>
+        <v>952729</v>
       </c>
       <c r="I691" s="6">
         <v>550540</v>
       </c>
       <c r="J691" s="6">
-        <v>3446</v>
+        <v>43859</v>
       </c>
       <c r="K691" s="6">
-        <v>553986</v>
+        <v>594399</v>
       </c>
       <c r="L691" s="6">
         <v>1465615</v>
       </c>
       <c r="M691" s="6">
-        <v>14295</v>
+        <v>81513</v>
       </c>
       <c r="N691" s="6">
-        <v>1479910</v>
+        <v>1547128</v>
       </c>
       <c r="O691" s="6">
-        <v>870675</v>
+        <v>897480</v>
       </c>
       <c r="P691" s="6">
         <v>51271</v>
@@ -57141,25 +57144,25 @@
         <v>78</v>
       </c>
       <c r="S691" s="6">
-        <v>925924</v>
+        <v>952729</v>
       </c>
       <c r="T691" s="6">
-        <v>497612</v>
+        <v>530582</v>
       </c>
       <c r="U691" s="6">
-        <v>52748</v>
+        <v>60129</v>
       </c>
       <c r="V691" s="6">
-        <v>3488</v>
+        <v>3580</v>
       </c>
       <c r="W691" s="6">
-        <v>138</v>
+        <v>108</v>
       </c>
       <c r="X691" s="6">
-        <v>553986</v>
+        <v>594399</v>
       </c>
       <c r="Y691" s="6">
-        <v>1479910</v>
+        <v>1547128</v>
       </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
@@ -57182,31 +57185,31 @@
         <v>937765</v>
       </c>
       <c r="G692" s="6">
-        <v>2917</v>
+        <v>10636</v>
       </c>
       <c r="H692" s="6">
-        <v>940682</v>
+        <v>948401</v>
       </c>
       <c r="I692" s="6">
         <v>445313</v>
       </c>
       <c r="J692" s="6">
-        <v>12763</v>
+        <v>15060</v>
       </c>
       <c r="K692" s="6">
-        <v>458076</v>
+        <v>460373</v>
       </c>
       <c r="L692" s="6">
         <v>1383078</v>
       </c>
       <c r="M692" s="6">
-        <v>15680</v>
+        <v>25696</v>
       </c>
       <c r="N692" s="6">
-        <v>1398758</v>
+        <v>1408774</v>
       </c>
       <c r="O692" s="6">
-        <v>876537</v>
+        <v>884256</v>
       </c>
       <c r="P692" s="6">
         <v>61445</v>
@@ -57218,13 +57221,13 @@
         <v>22</v>
       </c>
       <c r="S692" s="6">
-        <v>940682</v>
+        <v>948401</v>
       </c>
       <c r="T692" s="6">
-        <v>403146</v>
+        <v>405165</v>
       </c>
       <c r="U692" s="6">
-        <v>52163</v>
+        <v>52441</v>
       </c>
       <c r="V692" s="6">
         <v>2697</v>
@@ -57233,10 +57236,10 @@
         <v>70</v>
       </c>
       <c r="X692" s="6">
-        <v>458076</v>
+        <v>460373</v>
       </c>
       <c r="Y692" s="6">
-        <v>1398758</v>
+        <v>1408774</v>
       </c>
     </row>
     <row r="693" spans="1:25" x14ac:dyDescent="0.25">
@@ -57259,34 +57262,34 @@
         <v>800679</v>
       </c>
       <c r="G693" s="6">
-        <v>16871</v>
+        <v>19100</v>
       </c>
       <c r="H693" s="6">
-        <v>817550</v>
+        <v>819779</v>
       </c>
       <c r="I693" s="6">
         <v>343793</v>
       </c>
       <c r="J693" s="6">
-        <v>33956</v>
+        <v>36436</v>
       </c>
       <c r="K693" s="6">
-        <v>377749</v>
+        <v>380229</v>
       </c>
       <c r="L693" s="6">
         <v>1144472</v>
       </c>
       <c r="M693" s="6">
-        <v>50827</v>
+        <v>55536</v>
       </c>
       <c r="N693" s="6">
-        <v>1195299</v>
+        <v>1200008</v>
       </c>
       <c r="O693" s="6">
-        <v>751641</v>
+        <v>753842</v>
       </c>
       <c r="P693" s="6">
-        <v>62275</v>
+        <v>62303</v>
       </c>
       <c r="Q693" s="6">
         <v>3628</v>
@@ -57295,13 +57298,13 @@
         <v>6</v>
       </c>
       <c r="S693" s="6">
-        <v>817550</v>
+        <v>819779</v>
       </c>
       <c r="T693" s="6">
-        <v>336374</v>
+        <v>338668</v>
       </c>
       <c r="U693" s="6">
-        <v>40464</v>
+        <v>40650</v>
       </c>
       <c r="V693" s="6">
         <v>887</v>
@@ -57310,10 +57313,10 @@
         <v>24</v>
       </c>
       <c r="X693" s="6">
-        <v>377749</v>
+        <v>380229</v>
       </c>
       <c r="Y693" s="6">
-        <v>1195299</v>
+        <v>1200008</v>
       </c>
     </row>
     <row r="694" spans="1:25" x14ac:dyDescent="0.25">
@@ -57323,7 +57326,7 @@
       <c r="B694" s="4">
         <v>23</v>
       </c>
-      <c r="C694" s="60" t="s">
+      <c r="C694" s="59" t="s">
         <v>735</v>
       </c>
       <c r="D694" s="6" t="s">
@@ -57336,31 +57339,31 @@
         <v>637394</v>
       </c>
       <c r="G694" s="6">
-        <v>0</v>
+        <v>1102</v>
       </c>
       <c r="H694" s="6">
-        <v>637394</v>
+        <v>638496</v>
       </c>
       <c r="I694" s="6">
         <v>257890</v>
       </c>
       <c r="J694" s="6">
-        <v>0</v>
+        <v>574</v>
       </c>
       <c r="K694" s="6">
-        <v>257890</v>
+        <v>258464</v>
       </c>
       <c r="L694" s="6">
         <v>895284</v>
       </c>
       <c r="M694" s="6">
-        <v>0</v>
+        <v>1676</v>
       </c>
       <c r="N694" s="6">
-        <v>895284</v>
+        <v>896960</v>
       </c>
       <c r="O694" s="6">
-        <v>572666</v>
+        <v>573768</v>
       </c>
       <c r="P694" s="6">
         <v>61784</v>
@@ -57372,10 +57375,10 @@
         <v>26</v>
       </c>
       <c r="S694" s="6">
-        <v>637394</v>
+        <v>638496</v>
       </c>
       <c r="T694" s="6">
-        <v>228745</v>
+        <v>229319</v>
       </c>
       <c r="U694" s="6">
         <v>28327</v>
@@ -57387,10 +57390,10 @@
         <v>35</v>
       </c>
       <c r="X694" s="6">
-        <v>257890</v>
+        <v>258464</v>
       </c>
       <c r="Y694" s="6">
-        <v>895284</v>
+        <v>896960</v>
       </c>
     </row>
     <row r="695" spans="1:25" x14ac:dyDescent="0.25">
@@ -57400,33 +57403,75 @@
       <c r="B695" s="4">
         <v>24</v>
       </c>
-      <c r="C695" s="7"/>
+      <c r="C695" s="60" t="s">
+        <v>736</v>
+      </c>
       <c r="D695" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E695" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F695" s="6"/>
-      <c r="G695" s="6"/>
-      <c r="H695" s="6"/>
-      <c r="I695" s="6"/>
-      <c r="J695" s="6"/>
-      <c r="K695" s="6"/>
-      <c r="L695" s="6"/>
-      <c r="M695" s="6"/>
-      <c r="N695" s="6"/>
-      <c r="O695" s="6"/>
-      <c r="P695" s="6"/>
-      <c r="Q695" s="6"/>
-      <c r="R695" s="6"/>
-      <c r="S695" s="6"/>
-      <c r="T695" s="6"/>
-      <c r="U695" s="6"/>
-      <c r="V695" s="6"/>
-      <c r="W695" s="6"/>
-      <c r="X695" s="6"/>
-      <c r="Y695" s="6"/>
+      <c r="F695" s="6">
+        <v>268544</v>
+      </c>
+      <c r="G695" s="6">
+        <v>0</v>
+      </c>
+      <c r="H695" s="6">
+        <v>268544</v>
+      </c>
+      <c r="I695" s="6">
+        <v>85485</v>
+      </c>
+      <c r="J695" s="6">
+        <v>0</v>
+      </c>
+      <c r="K695" s="6">
+        <v>85485</v>
+      </c>
+      <c r="L695" s="6">
+        <v>354029</v>
+      </c>
+      <c r="M695" s="6">
+        <v>0</v>
+      </c>
+      <c r="N695" s="6">
+        <v>354029</v>
+      </c>
+      <c r="O695" s="6">
+        <v>236630</v>
+      </c>
+      <c r="P695" s="6">
+        <v>29987</v>
+      </c>
+      <c r="Q695" s="6">
+        <v>1923</v>
+      </c>
+      <c r="R695" s="6">
+        <v>4</v>
+      </c>
+      <c r="S695" s="6">
+        <v>268544</v>
+      </c>
+      <c r="T695" s="6">
+        <v>79032</v>
+      </c>
+      <c r="U695" s="6">
+        <v>6063</v>
+      </c>
+      <c r="V695" s="6">
+        <v>86</v>
+      </c>
+      <c r="W695" s="6">
+        <v>304</v>
+      </c>
+      <c r="X695" s="6">
+        <v>85485</v>
+      </c>
+      <c r="Y695" s="6">
+        <v>354029</v>
+      </c>
     </row>
     <row r="696" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A696" s="7">
@@ -58678,6 +58723,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -58904,17 +58960,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -58925,6 +58970,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
+    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -58943,17 +58999,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
-    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update AGR and deliveries through August 25
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{538A65DB-1B84-44A0-B0D1-8097CA8570A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D82071-17A8-470E-8B8B-7CDCD3C68742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16335" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2189" uniqueCount="737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2190" uniqueCount="738">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2247,6 +2247,9 @@
   </si>
   <si>
     <t>08/08 - 14/08/2026</t>
+  </si>
+  <si>
+    <t>15/08 - 21/08/2026</t>
   </si>
 </sst>
 </file>
@@ -54627,10 +54630,10 @@
         <v>18834</v>
       </c>
       <c r="G659" s="10">
-        <v>2115</v>
+        <v>2114</v>
       </c>
       <c r="H659" s="10">
-        <v>20949</v>
+        <v>20948</v>
       </c>
       <c r="I659" s="10">
         <v>22629</v>
@@ -54645,13 +54648,13 @@
         <v>41463</v>
       </c>
       <c r="M659" s="10">
-        <v>2154</v>
+        <v>2153</v>
       </c>
       <c r="N659" s="10">
-        <v>43617</v>
+        <v>43616</v>
       </c>
       <c r="O659" s="10">
-        <v>18370</v>
+        <v>18369</v>
       </c>
       <c r="P659" s="10">
         <v>2470</v>
@@ -54663,7 +54666,7 @@
         <v>0</v>
       </c>
       <c r="S659" s="10">
-        <v>20949</v>
+        <v>20948</v>
       </c>
       <c r="T659" s="10">
         <v>19705</v>
@@ -54681,7 +54684,7 @@
         <v>22668</v>
       </c>
       <c r="Y659" s="10">
-        <v>43617</v>
+        <v>43616</v>
       </c>
     </row>
     <row r="660" spans="1:27" x14ac:dyDescent="0.25">
@@ -56019,10 +56022,10 @@
         <v>42711</v>
       </c>
       <c r="G677" s="10">
-        <v>1790</v>
+        <v>1759</v>
       </c>
       <c r="H677" s="10">
-        <v>44501</v>
+        <v>44470</v>
       </c>
       <c r="I677" s="10">
         <v>60690</v>
@@ -56037,13 +56040,13 @@
         <v>103401</v>
       </c>
       <c r="M677" s="10">
-        <v>4792</v>
+        <v>4761</v>
       </c>
       <c r="N677" s="10">
-        <v>108193</v>
+        <v>108162</v>
       </c>
       <c r="O677" s="10">
-        <v>41773</v>
+        <v>41742</v>
       </c>
       <c r="P677" s="10">
         <v>2451</v>
@@ -56055,7 +56058,7 @@
         <v>87</v>
       </c>
       <c r="S677" s="10">
-        <v>44501</v>
+        <v>44470</v>
       </c>
       <c r="T677" s="10">
         <v>62135</v>
@@ -56073,7 +56076,7 @@
         <v>63692</v>
       </c>
       <c r="Y677" s="10">
-        <v>108193</v>
+        <v>108162</v>
       </c>
       <c r="AA677" s="57"/>
     </row>
@@ -56106,19 +56109,19 @@
         <v>79707</v>
       </c>
       <c r="J678" s="10">
-        <v>3200</v>
+        <v>3010</v>
       </c>
       <c r="K678" s="10">
-        <v>82907</v>
+        <v>82717</v>
       </c>
       <c r="L678" s="10">
         <v>132462</v>
       </c>
       <c r="M678" s="10">
-        <v>5829</v>
+        <v>5639</v>
       </c>
       <c r="N678" s="10">
-        <v>138291</v>
+        <v>138101</v>
       </c>
       <c r="O678" s="10">
         <v>51157</v>
@@ -56136,7 +56139,7 @@
         <v>55384</v>
       </c>
       <c r="T678" s="10">
-        <v>78366</v>
+        <v>78176</v>
       </c>
       <c r="U678" s="10">
         <v>4480</v>
@@ -56148,10 +56151,10 @@
         <v>61</v>
       </c>
       <c r="X678" s="10">
-        <v>82907</v>
+        <v>82717</v>
       </c>
       <c r="Y678" s="10">
-        <v>138291</v>
+        <v>138101</v>
       </c>
       <c r="AA678" s="57"/>
     </row>
@@ -56175,31 +56178,31 @@
         <v>31838</v>
       </c>
       <c r="G679" s="10">
-        <v>35859</v>
+        <v>35354</v>
       </c>
       <c r="H679" s="10">
-        <v>67697</v>
+        <v>67192</v>
       </c>
       <c r="I679" s="10">
         <v>74815</v>
       </c>
       <c r="J679" s="10">
-        <v>66951</v>
+        <v>66464</v>
       </c>
       <c r="K679" s="10">
-        <v>141766</v>
+        <v>141279</v>
       </c>
       <c r="L679" s="10">
         <v>106653</v>
       </c>
       <c r="M679" s="10">
-        <v>102810</v>
+        <v>101818</v>
       </c>
       <c r="N679" s="10">
-        <v>209463</v>
+        <v>208471</v>
       </c>
       <c r="O679" s="10">
-        <v>64972</v>
+        <v>64467</v>
       </c>
       <c r="P679" s="10">
         <v>1962</v>
@@ -56211,10 +56214,10 @@
         <v>87</v>
       </c>
       <c r="S679" s="10">
-        <v>67697</v>
+        <v>67192</v>
       </c>
       <c r="T679" s="10">
-        <v>138452</v>
+        <v>137965</v>
       </c>
       <c r="U679" s="10">
         <v>3296</v>
@@ -56226,10 +56229,10 @@
         <v>18</v>
       </c>
       <c r="X679" s="10">
-        <v>141766</v>
+        <v>141279</v>
       </c>
       <c r="Y679" s="10">
-        <v>209463</v>
+        <v>208471</v>
       </c>
       <c r="AA679" s="57"/>
     </row>
@@ -56262,19 +56265,19 @@
         <v>67676</v>
       </c>
       <c r="J680" s="16">
-        <v>-58015</v>
+        <v>-57174</v>
       </c>
       <c r="K680" s="16">
-        <v>9661</v>
+        <v>10502</v>
       </c>
       <c r="L680" s="16">
         <v>95738</v>
       </c>
       <c r="M680" s="16">
-        <v>-82070</v>
+        <v>-81229</v>
       </c>
       <c r="N680" s="16">
-        <v>13668</v>
+        <v>14509</v>
       </c>
       <c r="O680" s="16">
         <v>3577</v>
@@ -56292,7 +56295,7 @@
         <v>4007</v>
       </c>
       <c r="T680" s="16">
-        <v>9538</v>
+        <v>10379</v>
       </c>
       <c r="U680" s="16">
         <v>123</v>
@@ -56304,10 +56307,10 @@
         <v>0</v>
       </c>
       <c r="X680" s="16">
-        <v>9661</v>
+        <v>10502</v>
       </c>
       <c r="Y680" s="16">
-        <v>13668</v>
+        <v>14509</v>
       </c>
       <c r="Z680" s="19"/>
       <c r="AA680" s="57"/>
@@ -56332,10 +56335,10 @@
         <v>28999</v>
       </c>
       <c r="G681" s="10">
-        <v>476</v>
+        <v>1559</v>
       </c>
       <c r="H681" s="10">
-        <v>29475</v>
+        <v>30558</v>
       </c>
       <c r="I681" s="10">
         <v>73014</v>
@@ -56350,13 +56353,13 @@
         <v>102013</v>
       </c>
       <c r="M681" s="10">
-        <v>861</v>
+        <v>1944</v>
       </c>
       <c r="N681" s="10">
-        <v>102874</v>
+        <v>103957</v>
       </c>
       <c r="O681" s="10">
-        <v>27562</v>
+        <v>28645</v>
       </c>
       <c r="P681" s="10">
         <v>1766</v>
@@ -56368,7 +56371,7 @@
         <v>91</v>
       </c>
       <c r="S681" s="10">
-        <v>29475</v>
+        <v>30558</v>
       </c>
       <c r="T681" s="10">
         <v>72084</v>
@@ -56386,7 +56389,7 @@
         <v>73399</v>
       </c>
       <c r="Y681" s="10">
-        <v>102874</v>
+        <v>103957</v>
       </c>
       <c r="AA681" s="57"/>
     </row>
@@ -56410,34 +56413,34 @@
         <v>67674</v>
       </c>
       <c r="G682" s="10">
-        <v>154</v>
+        <v>512</v>
       </c>
       <c r="H682" s="10">
-        <v>67828</v>
+        <v>68186</v>
       </c>
       <c r="I682" s="10">
         <v>137597</v>
       </c>
       <c r="J682" s="10">
-        <v>2480</v>
+        <v>3365</v>
       </c>
       <c r="K682" s="10">
-        <v>140077</v>
+        <v>140962</v>
       </c>
       <c r="L682" s="10">
         <v>205271</v>
       </c>
       <c r="M682" s="10">
-        <v>2634</v>
+        <v>3877</v>
       </c>
       <c r="N682" s="10">
-        <v>207905</v>
+        <v>209148</v>
       </c>
       <c r="O682" s="10">
-        <v>63822</v>
+        <v>64145</v>
       </c>
       <c r="P682" s="10">
-        <v>3933</v>
+        <v>3968</v>
       </c>
       <c r="Q682" s="10">
         <v>35</v>
@@ -56446,10 +56449,10 @@
         <v>38</v>
       </c>
       <c r="S682" s="10">
-        <v>67828</v>
+        <v>68186</v>
       </c>
       <c r="T682" s="10">
-        <v>137076</v>
+        <v>137961</v>
       </c>
       <c r="U682" s="10">
         <v>2859</v>
@@ -56461,10 +56464,10 @@
         <v>37</v>
       </c>
       <c r="X682" s="10">
-        <v>140077</v>
+        <v>140962</v>
       </c>
       <c r="Y682" s="10">
-        <v>207905</v>
+        <v>209148</v>
       </c>
       <c r="AA682" s="57"/>
     </row>
@@ -56488,34 +56491,34 @@
         <v>120859</v>
       </c>
       <c r="G683" s="10">
-        <v>-193</v>
+        <v>803</v>
       </c>
       <c r="H683" s="10">
-        <v>120666</v>
+        <v>121662</v>
       </c>
       <c r="I683" s="10">
         <v>285962</v>
       </c>
       <c r="J683" s="10">
-        <v>2860</v>
+        <v>3688</v>
       </c>
       <c r="K683" s="10">
-        <v>288822</v>
+        <v>289650</v>
       </c>
       <c r="L683" s="10">
         <v>406821</v>
       </c>
       <c r="M683" s="10">
-        <v>2667</v>
+        <v>4491</v>
       </c>
       <c r="N683" s="10">
-        <v>409488</v>
+        <v>411312</v>
       </c>
       <c r="O683" s="10">
-        <v>115619</v>
+        <v>116369</v>
       </c>
       <c r="P683" s="10">
-        <v>4216</v>
+        <v>4462</v>
       </c>
       <c r="Q683" s="10">
         <v>720</v>
@@ -56524,10 +56527,10 @@
         <v>111</v>
       </c>
       <c r="S683" s="10">
-        <v>120666</v>
+        <v>121662</v>
       </c>
       <c r="T683" s="10">
-        <v>277464</v>
+        <v>278292</v>
       </c>
       <c r="U683" s="10">
         <v>10777</v>
@@ -56539,10 +56542,10 @@
         <v>2</v>
       </c>
       <c r="X683" s="10">
-        <v>288822</v>
+        <v>289650</v>
       </c>
       <c r="Y683" s="10">
-        <v>409488</v>
+        <v>411312</v>
       </c>
       <c r="AA683" s="57"/>
     </row>
@@ -56566,34 +56569,34 @@
         <v>201415</v>
       </c>
       <c r="G684" s="10">
-        <v>11275</v>
+        <v>12682</v>
       </c>
       <c r="H684" s="10">
-        <v>212690</v>
+        <v>214097</v>
       </c>
       <c r="I684" s="10">
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>34205</v>
+        <v>31357</v>
       </c>
       <c r="K684" s="10">
-        <v>447064</v>
+        <v>444216</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>45480</v>
+        <v>44039</v>
       </c>
       <c r="N684" s="10">
-        <v>659754</v>
+        <v>658313</v>
       </c>
       <c r="O684" s="10">
-        <v>203773</v>
+        <v>205162</v>
       </c>
       <c r="P684" s="10">
-        <v>8021</v>
+        <v>8039</v>
       </c>
       <c r="Q684" s="10">
         <v>761</v>
@@ -56602,10 +56605,10 @@
         <v>135</v>
       </c>
       <c r="S684" s="10">
-        <v>212690</v>
+        <v>214097</v>
       </c>
       <c r="T684" s="10">
-        <v>423314</v>
+        <v>420466</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56617,10 +56620,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>447064</v>
+        <v>444216</v>
       </c>
       <c r="Y684" s="10">
-        <v>659754</v>
+        <v>658313</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56644,10 +56647,10 @@
         <v>290878</v>
       </c>
       <c r="G685" s="10">
-        <v>1711</v>
+        <v>1367</v>
       </c>
       <c r="H685" s="10">
-        <v>292589</v>
+        <v>292245</v>
       </c>
       <c r="I685" s="10">
         <v>435387</v>
@@ -56662,13 +56665,13 @@
         <v>726265</v>
       </c>
       <c r="M685" s="10">
-        <v>16840</v>
+        <v>16496</v>
       </c>
       <c r="N685" s="10">
-        <v>743105</v>
+        <v>742761</v>
       </c>
       <c r="O685" s="10">
-        <v>276060</v>
+        <v>275716</v>
       </c>
       <c r="P685" s="10">
         <v>15443</v>
@@ -56680,7 +56683,7 @@
         <v>69</v>
       </c>
       <c r="S685" s="10">
-        <v>292589</v>
+        <v>292245</v>
       </c>
       <c r="T685" s="10">
         <v>414816</v>
@@ -56698,7 +56701,7 @@
         <v>450516</v>
       </c>
       <c r="Y685" s="10">
-        <v>743105</v>
+        <v>742761</v>
       </c>
       <c r="AA685" s="57"/>
     </row>
@@ -56800,10 +56803,10 @@
         <v>702695</v>
       </c>
       <c r="G687" s="6">
-        <v>8369</v>
+        <v>8199</v>
       </c>
       <c r="H687" s="6">
-        <v>711064</v>
+        <v>710894</v>
       </c>
       <c r="I687" s="6">
         <v>669414</v>
@@ -56818,13 +56821,13 @@
         <v>1372109</v>
       </c>
       <c r="M687" s="6">
-        <v>14713</v>
+        <v>14543</v>
       </c>
       <c r="N687" s="6">
-        <v>1386822</v>
+        <v>1386652</v>
       </c>
       <c r="O687" s="6">
-        <v>674414</v>
+        <v>674244</v>
       </c>
       <c r="P687" s="6">
         <v>34795</v>
@@ -56836,7 +56839,7 @@
         <v>45</v>
       </c>
       <c r="S687" s="6">
-        <v>711064</v>
+        <v>710894</v>
       </c>
       <c r="T687" s="6">
         <v>614475</v>
@@ -56854,7 +56857,7 @@
         <v>675758</v>
       </c>
       <c r="Y687" s="6">
-        <v>1386822</v>
+        <v>1386652</v>
       </c>
     </row>
     <row r="688" spans="1:27" x14ac:dyDescent="0.25">
@@ -56877,31 +56880,31 @@
         <v>456498</v>
       </c>
       <c r="G688" s="6">
-        <v>46724</v>
+        <v>46223</v>
       </c>
       <c r="H688" s="6">
-        <v>503222</v>
+        <v>502721</v>
       </c>
       <c r="I688" s="6">
         <v>390877</v>
       </c>
       <c r="J688" s="6">
-        <v>74793</v>
+        <v>75154</v>
       </c>
       <c r="K688" s="6">
-        <v>465670</v>
+        <v>466031</v>
       </c>
       <c r="L688" s="6">
         <v>847375</v>
       </c>
       <c r="M688" s="6">
-        <v>121517</v>
+        <v>121377</v>
       </c>
       <c r="N688" s="6">
-        <v>968892</v>
+        <v>968752</v>
       </c>
       <c r="O688" s="6">
-        <v>475972</v>
+        <v>475471</v>
       </c>
       <c r="P688" s="6">
         <v>24451</v>
@@ -56913,10 +56916,10 @@
         <v>36</v>
       </c>
       <c r="S688" s="6">
-        <v>503222</v>
+        <v>502721</v>
       </c>
       <c r="T688" s="6">
-        <v>433119</v>
+        <v>433480</v>
       </c>
       <c r="U688" s="6">
         <v>31539</v>
@@ -56928,10 +56931,10 @@
         <v>188</v>
       </c>
       <c r="X688" s="6">
-        <v>465670</v>
+        <v>466031</v>
       </c>
       <c r="Y688" s="6">
-        <v>968892</v>
+        <v>968752</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -56954,46 +56957,46 @@
         <v>488226</v>
       </c>
       <c r="G689" s="6">
-        <v>6304</v>
+        <v>31095</v>
       </c>
       <c r="H689" s="6">
-        <v>494530</v>
+        <v>519321</v>
       </c>
       <c r="I689" s="6">
         <v>379489</v>
       </c>
       <c r="J689" s="6">
-        <v>13355</v>
+        <v>13267</v>
       </c>
       <c r="K689" s="6">
-        <v>392844</v>
+        <v>392756</v>
       </c>
       <c r="L689" s="6">
         <v>867715</v>
       </c>
       <c r="M689" s="6">
-        <v>19659</v>
+        <v>44362</v>
       </c>
       <c r="N689" s="6">
-        <v>887374</v>
+        <v>912077</v>
       </c>
       <c r="O689" s="6">
-        <v>465998</v>
+        <v>490124</v>
       </c>
       <c r="P689" s="6">
-        <v>25603</v>
+        <v>26156</v>
       </c>
       <c r="Q689" s="6">
-        <v>2884</v>
+        <v>2991</v>
       </c>
       <c r="R689" s="6">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="S689" s="6">
-        <v>494530</v>
+        <v>519321</v>
       </c>
       <c r="T689" s="6">
-        <v>358168</v>
+        <v>358080</v>
       </c>
       <c r="U689" s="6">
         <v>33163</v>
@@ -57005,10 +57008,10 @@
         <v>70</v>
       </c>
       <c r="X689" s="6">
-        <v>392844</v>
+        <v>392756</v>
       </c>
       <c r="Y689" s="6">
-        <v>887374</v>
+        <v>912077</v>
       </c>
     </row>
     <row r="690" spans="1:25" x14ac:dyDescent="0.25">
@@ -57031,34 +57034,34 @@
         <v>833175</v>
       </c>
       <c r="G690" s="6">
-        <v>9035</v>
+        <v>9096</v>
       </c>
       <c r="H690" s="6">
-        <v>842210</v>
+        <v>842271</v>
       </c>
       <c r="I690" s="6">
         <v>556930</v>
       </c>
       <c r="J690" s="6">
-        <v>6465</v>
+        <v>6087</v>
       </c>
       <c r="K690" s="6">
-        <v>563395</v>
+        <v>563017</v>
       </c>
       <c r="L690" s="6">
         <v>1390105</v>
       </c>
       <c r="M690" s="6">
-        <v>15500</v>
+        <v>15183</v>
       </c>
       <c r="N690" s="6">
-        <v>1405605</v>
+        <v>1405288</v>
       </c>
       <c r="O690" s="6">
-        <v>794603</v>
+        <v>794565</v>
       </c>
       <c r="P690" s="6">
-        <v>42085</v>
+        <v>42184</v>
       </c>
       <c r="Q690" s="6">
         <v>5458</v>
@@ -57067,10 +57070,10 @@
         <v>64</v>
       </c>
       <c r="S690" s="6">
-        <v>842210</v>
+        <v>842271</v>
       </c>
       <c r="T690" s="6">
-        <v>502494</v>
+        <v>502116</v>
       </c>
       <c r="U690" s="6">
         <v>58757</v>
@@ -57082,10 +57085,10 @@
         <v>131</v>
       </c>
       <c r="X690" s="6">
-        <v>563395</v>
+        <v>563017</v>
       </c>
       <c r="Y690" s="6">
-        <v>1405605</v>
+        <v>1405288</v>
       </c>
     </row>
     <row r="691" spans="1:25" x14ac:dyDescent="0.25">
@@ -57108,46 +57111,46 @@
         <v>915075</v>
       </c>
       <c r="G691" s="6">
-        <v>37654</v>
+        <v>59510</v>
       </c>
       <c r="H691" s="6">
-        <v>952729</v>
+        <v>974585</v>
       </c>
       <c r="I691" s="6">
         <v>550540</v>
       </c>
       <c r="J691" s="6">
-        <v>43859</v>
+        <v>43860</v>
       </c>
       <c r="K691" s="6">
-        <v>594399</v>
+        <v>594400</v>
       </c>
       <c r="L691" s="6">
         <v>1465615</v>
       </c>
       <c r="M691" s="6">
-        <v>81513</v>
+        <v>103370</v>
       </c>
       <c r="N691" s="6">
-        <v>1547128</v>
+        <v>1568985</v>
       </c>
       <c r="O691" s="6">
-        <v>897480</v>
+        <v>911320</v>
       </c>
       <c r="P691" s="6">
-        <v>51271</v>
+        <v>58498</v>
       </c>
       <c r="Q691" s="6">
-        <v>3900</v>
+        <v>4689</v>
       </c>
       <c r="R691" s="6">
         <v>78</v>
       </c>
       <c r="S691" s="6">
-        <v>952729</v>
+        <v>974585</v>
       </c>
       <c r="T691" s="6">
-        <v>530582</v>
+        <v>530583</v>
       </c>
       <c r="U691" s="6">
         <v>60129</v>
@@ -57159,10 +57162,10 @@
         <v>108</v>
       </c>
       <c r="X691" s="6">
-        <v>594399</v>
+        <v>594400</v>
       </c>
       <c r="Y691" s="6">
-        <v>1547128</v>
+        <v>1568985</v>
       </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
@@ -57185,34 +57188,34 @@
         <v>937765</v>
       </c>
       <c r="G692" s="6">
-        <v>10636</v>
+        <v>10681</v>
       </c>
       <c r="H692" s="6">
-        <v>948401</v>
+        <v>948446</v>
       </c>
       <c r="I692" s="6">
         <v>445313</v>
       </c>
       <c r="J692" s="6">
-        <v>15060</v>
+        <v>15559</v>
       </c>
       <c r="K692" s="6">
-        <v>460373</v>
+        <v>460872</v>
       </c>
       <c r="L692" s="6">
         <v>1383078</v>
       </c>
       <c r="M692" s="6">
-        <v>25696</v>
+        <v>26240</v>
       </c>
       <c r="N692" s="6">
-        <v>1408774</v>
+        <v>1409318</v>
       </c>
       <c r="O692" s="6">
-        <v>884256</v>
+        <v>884230</v>
       </c>
       <c r="P692" s="6">
-        <v>61445</v>
+        <v>61516</v>
       </c>
       <c r="Q692" s="6">
         <v>2678</v>
@@ -57221,13 +57224,13 @@
         <v>22</v>
       </c>
       <c r="S692" s="6">
-        <v>948401</v>
+        <v>948446</v>
       </c>
       <c r="T692" s="6">
-        <v>405165</v>
+        <v>405590</v>
       </c>
       <c r="U692" s="6">
-        <v>52441</v>
+        <v>52515</v>
       </c>
       <c r="V692" s="6">
         <v>2697</v>
@@ -57236,10 +57239,10 @@
         <v>70</v>
       </c>
       <c r="X692" s="6">
-        <v>460373</v>
+        <v>460872</v>
       </c>
       <c r="Y692" s="6">
-        <v>1408774</v>
+        <v>1409318</v>
       </c>
     </row>
     <row r="693" spans="1:25" x14ac:dyDescent="0.25">
@@ -57262,31 +57265,31 @@
         <v>800679</v>
       </c>
       <c r="G693" s="6">
-        <v>19100</v>
+        <v>56421</v>
       </c>
       <c r="H693" s="6">
-        <v>819779</v>
+        <v>857100</v>
       </c>
       <c r="I693" s="6">
         <v>343793</v>
       </c>
       <c r="J693" s="6">
-        <v>36436</v>
+        <v>75807</v>
       </c>
       <c r="K693" s="6">
-        <v>380229</v>
+        <v>419600</v>
       </c>
       <c r="L693" s="6">
         <v>1144472</v>
       </c>
       <c r="M693" s="6">
-        <v>55536</v>
+        <v>132228</v>
       </c>
       <c r="N693" s="6">
-        <v>1200008</v>
+        <v>1276700</v>
       </c>
       <c r="O693" s="6">
-        <v>753842</v>
+        <v>791163</v>
       </c>
       <c r="P693" s="6">
         <v>62303</v>
@@ -57298,13 +57301,13 @@
         <v>6</v>
       </c>
       <c r="S693" s="6">
-        <v>819779</v>
+        <v>857100</v>
       </c>
       <c r="T693" s="6">
-        <v>338668</v>
+        <v>378007</v>
       </c>
       <c r="U693" s="6">
-        <v>40650</v>
+        <v>40682</v>
       </c>
       <c r="V693" s="6">
         <v>887</v>
@@ -57313,10 +57316,10 @@
         <v>24</v>
       </c>
       <c r="X693" s="6">
-        <v>380229</v>
+        <v>419600</v>
       </c>
       <c r="Y693" s="6">
-        <v>1200008</v>
+        <v>1276700</v>
       </c>
     </row>
     <row r="694" spans="1:25" x14ac:dyDescent="0.25">
@@ -57339,31 +57342,31 @@
         <v>637394</v>
       </c>
       <c r="G694" s="6">
-        <v>1102</v>
+        <v>1241</v>
       </c>
       <c r="H694" s="6">
-        <v>638496</v>
+        <v>638635</v>
       </c>
       <c r="I694" s="6">
         <v>257890</v>
       </c>
       <c r="J694" s="6">
-        <v>574</v>
+        <v>1542</v>
       </c>
       <c r="K694" s="6">
-        <v>258464</v>
+        <v>259432</v>
       </c>
       <c r="L694" s="6">
         <v>895284</v>
       </c>
       <c r="M694" s="6">
-        <v>1676</v>
+        <v>2783</v>
       </c>
       <c r="N694" s="6">
-        <v>896960</v>
+        <v>898067</v>
       </c>
       <c r="O694" s="6">
-        <v>573768</v>
+        <v>573907</v>
       </c>
       <c r="P694" s="6">
         <v>61784</v>
@@ -57375,10 +57378,10 @@
         <v>26</v>
       </c>
       <c r="S694" s="6">
-        <v>638496</v>
+        <v>638635</v>
       </c>
       <c r="T694" s="6">
-        <v>229319</v>
+        <v>230287</v>
       </c>
       <c r="U694" s="6">
         <v>28327</v>
@@ -57390,10 +57393,10 @@
         <v>35</v>
       </c>
       <c r="X694" s="6">
-        <v>258464</v>
+        <v>259432</v>
       </c>
       <c r="Y694" s="6">
-        <v>896960</v>
+        <v>898067</v>
       </c>
     </row>
     <row r="695" spans="1:25" x14ac:dyDescent="0.25">
@@ -57403,7 +57406,7 @@
       <c r="B695" s="4">
         <v>24</v>
       </c>
-      <c r="C695" s="60" t="s">
+      <c r="C695" s="59" t="s">
         <v>736</v>
       </c>
       <c r="D695" s="6" t="s">
@@ -57416,34 +57419,34 @@
         <v>268544</v>
       </c>
       <c r="G695" s="6">
-        <v>0</v>
+        <v>618</v>
       </c>
       <c r="H695" s="6">
-        <v>268544</v>
+        <v>269162</v>
       </c>
       <c r="I695" s="6">
         <v>85485</v>
       </c>
       <c r="J695" s="6">
-        <v>0</v>
+        <v>1070</v>
       </c>
       <c r="K695" s="6">
-        <v>85485</v>
+        <v>86555</v>
       </c>
       <c r="L695" s="6">
         <v>354029</v>
       </c>
       <c r="M695" s="6">
-        <v>0</v>
+        <v>1688</v>
       </c>
       <c r="N695" s="6">
-        <v>354029</v>
+        <v>355717</v>
       </c>
       <c r="O695" s="6">
-        <v>236630</v>
+        <v>237149</v>
       </c>
       <c r="P695" s="6">
-        <v>29987</v>
+        <v>30086</v>
       </c>
       <c r="Q695" s="6">
         <v>1923</v>
@@ -57452,13 +57455,13 @@
         <v>4</v>
       </c>
       <c r="S695" s="6">
-        <v>268544</v>
+        <v>269162</v>
       </c>
       <c r="T695" s="6">
-        <v>79032</v>
+        <v>80033</v>
       </c>
       <c r="U695" s="6">
-        <v>6063</v>
+        <v>6132</v>
       </c>
       <c r="V695" s="6">
         <v>86</v>
@@ -57467,10 +57470,10 @@
         <v>304</v>
       </c>
       <c r="X695" s="6">
-        <v>85485</v>
+        <v>86555</v>
       </c>
       <c r="Y695" s="6">
-        <v>354029</v>
+        <v>355717</v>
       </c>
     </row>
     <row r="696" spans="1:25" x14ac:dyDescent="0.25">
@@ -57480,33 +57483,75 @@
       <c r="B696" s="4">
         <v>25</v>
       </c>
-      <c r="C696" s="7"/>
+      <c r="C696" s="60" t="s">
+        <v>737</v>
+      </c>
       <c r="D696" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E696" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F696" s="6"/>
-      <c r="G696" s="6"/>
-      <c r="H696" s="6"/>
-      <c r="I696" s="6"/>
-      <c r="J696" s="6"/>
-      <c r="K696" s="6"/>
-      <c r="L696" s="6"/>
-      <c r="M696" s="6"/>
-      <c r="N696" s="6"/>
-      <c r="O696" s="6"/>
-      <c r="P696" s="6"/>
-      <c r="Q696" s="6"/>
-      <c r="R696" s="6"/>
-      <c r="S696" s="6"/>
-      <c r="T696" s="6"/>
-      <c r="U696" s="6"/>
-      <c r="V696" s="6"/>
-      <c r="W696" s="6"/>
-      <c r="X696" s="6"/>
-      <c r="Y696" s="6"/>
+      <c r="F696" s="6">
+        <v>432804</v>
+      </c>
+      <c r="G696" s="6">
+        <v>0</v>
+      </c>
+      <c r="H696" s="6">
+        <v>432804</v>
+      </c>
+      <c r="I696" s="6">
+        <v>150038</v>
+      </c>
+      <c r="J696" s="6">
+        <v>0</v>
+      </c>
+      <c r="K696" s="6">
+        <v>150038</v>
+      </c>
+      <c r="L696" s="6">
+        <v>582842</v>
+      </c>
+      <c r="M696" s="6">
+        <v>0</v>
+      </c>
+      <c r="N696" s="6">
+        <v>582842</v>
+      </c>
+      <c r="O696" s="6">
+        <v>379826</v>
+      </c>
+      <c r="P696" s="6">
+        <v>48627</v>
+      </c>
+      <c r="Q696" s="6">
+        <v>4323</v>
+      </c>
+      <c r="R696" s="6">
+        <v>28</v>
+      </c>
+      <c r="S696" s="6">
+        <v>432804</v>
+      </c>
+      <c r="T696" s="6">
+        <v>134150</v>
+      </c>
+      <c r="U696" s="6">
+        <v>15007</v>
+      </c>
+      <c r="V696" s="6">
+        <v>874</v>
+      </c>
+      <c r="W696" s="6">
+        <v>7</v>
+      </c>
+      <c r="X696" s="6">
+        <v>150038</v>
+      </c>
+      <c r="Y696" s="6">
+        <v>582842</v>
+      </c>
     </row>
     <row r="697" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A697" s="7">

</xml_diff>

<commit_message>
Update AGR and deliveries data through September 1
</commit_message>
<xml_diff>
--- a/Clean_deliveries_format_maize.xlsx
+++ b/Clean_deliveries_format_maize.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\grain-data-intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D82071-17A8-470E-8B8B-7CDCD3C68742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49EF237-9C23-42B4-935C-79440287D738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16335" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-16200" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2190" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2191" uniqueCount="739">
   <si>
     <t>SAGIS Week nr</t>
   </si>
@@ -2250,6 +2250,9 @@
   </si>
   <si>
     <t>15/08 - 21/08/2026</t>
+  </si>
+  <si>
+    <t>22/08 - 28/08/2026</t>
   </si>
 </sst>
 </file>
@@ -4531,14 +4534,14 @@
         <v>77</v>
       </c>
       <c r="AD16" s="51">
-        <v>9390790</v>
+        <v>9487790</v>
       </c>
       <c r="AE16" s="51">
-        <v>7971850</v>
+        <v>7914050</v>
       </c>
       <c r="AF16" s="53">
         <f>AE16+AD16</f>
-        <v>17362640</v>
+        <v>17401840</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
@@ -56578,19 +56581,19 @@
         <v>412859</v>
       </c>
       <c r="J684" s="10">
-        <v>31357</v>
+        <v>31474</v>
       </c>
       <c r="K684" s="10">
-        <v>444216</v>
+        <v>444333</v>
       </c>
       <c r="L684" s="10">
         <v>614274</v>
       </c>
       <c r="M684" s="10">
-        <v>44039</v>
+        <v>44156</v>
       </c>
       <c r="N684" s="10">
-        <v>658313</v>
+        <v>658430</v>
       </c>
       <c r="O684" s="10">
         <v>205162</v>
@@ -56608,7 +56611,7 @@
         <v>214097</v>
       </c>
       <c r="T684" s="10">
-        <v>420466</v>
+        <v>420583</v>
       </c>
       <c r="U684" s="10">
         <v>23148</v>
@@ -56620,10 +56623,10 @@
         <v>47</v>
       </c>
       <c r="X684" s="10">
-        <v>444216</v>
+        <v>444333</v>
       </c>
       <c r="Y684" s="10">
-        <v>658313</v>
+        <v>658430</v>
       </c>
       <c r="AA684" s="57"/>
     </row>
@@ -56803,10 +56806,10 @@
         <v>702695</v>
       </c>
       <c r="G687" s="6">
-        <v>8199</v>
+        <v>8754</v>
       </c>
       <c r="H687" s="6">
-        <v>710894</v>
+        <v>711449</v>
       </c>
       <c r="I687" s="6">
         <v>669414</v>
@@ -56821,13 +56824,13 @@
         <v>1372109</v>
       </c>
       <c r="M687" s="6">
-        <v>14543</v>
+        <v>15098</v>
       </c>
       <c r="N687" s="6">
-        <v>1386652</v>
+        <v>1387207</v>
       </c>
       <c r="O687" s="6">
-        <v>674244</v>
+        <v>674799</v>
       </c>
       <c r="P687" s="6">
         <v>34795</v>
@@ -56839,7 +56842,7 @@
         <v>45</v>
       </c>
       <c r="S687" s="6">
-        <v>710894</v>
+        <v>711449</v>
       </c>
       <c r="T687" s="6">
         <v>614475</v>
@@ -56857,7 +56860,7 @@
         <v>675758</v>
       </c>
       <c r="Y687" s="6">
-        <v>1386652</v>
+        <v>1387207</v>
       </c>
     </row>
     <row r="688" spans="1:27" x14ac:dyDescent="0.25">
@@ -56880,31 +56883,31 @@
         <v>456498</v>
       </c>
       <c r="G688" s="6">
-        <v>46223</v>
+        <v>47110</v>
       </c>
       <c r="H688" s="6">
-        <v>502721</v>
+        <v>503608</v>
       </c>
       <c r="I688" s="6">
         <v>390877</v>
       </c>
       <c r="J688" s="6">
-        <v>75154</v>
+        <v>75176</v>
       </c>
       <c r="K688" s="6">
-        <v>466031</v>
+        <v>466053</v>
       </c>
       <c r="L688" s="6">
         <v>847375</v>
       </c>
       <c r="M688" s="6">
-        <v>121377</v>
+        <v>122286</v>
       </c>
       <c r="N688" s="6">
-        <v>968752</v>
+        <v>969661</v>
       </c>
       <c r="O688" s="6">
-        <v>475471</v>
+        <v>476358</v>
       </c>
       <c r="P688" s="6">
         <v>24451</v>
@@ -56916,10 +56919,10 @@
         <v>36</v>
       </c>
       <c r="S688" s="6">
-        <v>502721</v>
+        <v>503608</v>
       </c>
       <c r="T688" s="6">
-        <v>433480</v>
+        <v>433502</v>
       </c>
       <c r="U688" s="6">
         <v>31539</v>
@@ -56931,10 +56934,10 @@
         <v>188</v>
       </c>
       <c r="X688" s="6">
-        <v>466031</v>
+        <v>466053</v>
       </c>
       <c r="Y688" s="6">
-        <v>968752</v>
+        <v>969661</v>
       </c>
     </row>
     <row r="689" spans="1:25" x14ac:dyDescent="0.25">
@@ -56957,31 +56960,31 @@
         <v>488226</v>
       </c>
       <c r="G689" s="6">
-        <v>31095</v>
+        <v>33395</v>
       </c>
       <c r="H689" s="6">
-        <v>519321</v>
+        <v>521621</v>
       </c>
       <c r="I689" s="6">
         <v>379489</v>
       </c>
       <c r="J689" s="6">
-        <v>13267</v>
+        <v>13568</v>
       </c>
       <c r="K689" s="6">
-        <v>392756</v>
+        <v>393057</v>
       </c>
       <c r="L689" s="6">
         <v>867715</v>
       </c>
       <c r="M689" s="6">
-        <v>44362</v>
+        <v>46963</v>
       </c>
       <c r="N689" s="6">
-        <v>912077</v>
+        <v>914678</v>
       </c>
       <c r="O689" s="6">
-        <v>490124</v>
+        <v>492424</v>
       </c>
       <c r="P689" s="6">
         <v>26156</v>
@@ -56993,10 +56996,10 @@
         <v>50</v>
       </c>
       <c r="S689" s="6">
-        <v>519321</v>
+        <v>521621</v>
       </c>
       <c r="T689" s="6">
-        <v>358080</v>
+        <v>358381</v>
       </c>
       <c r="U689" s="6">
         <v>33163</v>
@@ -57008,10 +57011,10 @@
         <v>70</v>
       </c>
       <c r="X689" s="6">
-        <v>392756</v>
+        <v>393057</v>
       </c>
       <c r="Y689" s="6">
-        <v>912077</v>
+        <v>914678</v>
       </c>
     </row>
     <row r="690" spans="1:25" x14ac:dyDescent="0.25">
@@ -57034,31 +57037,31 @@
         <v>833175</v>
       </c>
       <c r="G690" s="6">
-        <v>9096</v>
+        <v>10521</v>
       </c>
       <c r="H690" s="6">
-        <v>842271</v>
+        <v>843696</v>
       </c>
       <c r="I690" s="6">
         <v>556930</v>
       </c>
       <c r="J690" s="6">
-        <v>6087</v>
+        <v>6584</v>
       </c>
       <c r="K690" s="6">
-        <v>563017</v>
+        <v>563514</v>
       </c>
       <c r="L690" s="6">
         <v>1390105</v>
       </c>
       <c r="M690" s="6">
-        <v>15183</v>
+        <v>17105</v>
       </c>
       <c r="N690" s="6">
-        <v>1405288</v>
+        <v>1407210</v>
       </c>
       <c r="O690" s="6">
-        <v>794565</v>
+        <v>795990</v>
       </c>
       <c r="P690" s="6">
         <v>42184</v>
@@ -57070,10 +57073,10 @@
         <v>64</v>
       </c>
       <c r="S690" s="6">
-        <v>842271</v>
+        <v>843696</v>
       </c>
       <c r="T690" s="6">
-        <v>502116</v>
+        <v>502613</v>
       </c>
       <c r="U690" s="6">
         <v>58757</v>
@@ -57085,10 +57088,10 @@
         <v>131</v>
       </c>
       <c r="X690" s="6">
-        <v>563017</v>
+        <v>563514</v>
       </c>
       <c r="Y690" s="6">
-        <v>1405288</v>
+        <v>1407210</v>
       </c>
     </row>
     <row r="691" spans="1:25" x14ac:dyDescent="0.25">
@@ -57111,31 +57114,31 @@
         <v>915075</v>
       </c>
       <c r="G691" s="6">
-        <v>59510</v>
+        <v>59905</v>
       </c>
       <c r="H691" s="6">
-        <v>974585</v>
+        <v>974980</v>
       </c>
       <c r="I691" s="6">
         <v>550540</v>
       </c>
       <c r="J691" s="6">
-        <v>43860</v>
+        <v>43925</v>
       </c>
       <c r="K691" s="6">
-        <v>594400</v>
+        <v>594465</v>
       </c>
       <c r="L691" s="6">
         <v>1465615</v>
       </c>
       <c r="M691" s="6">
-        <v>103370</v>
+        <v>103830</v>
       </c>
       <c r="N691" s="6">
-        <v>1568985</v>
+        <v>1569445</v>
       </c>
       <c r="O691" s="6">
-        <v>911320</v>
+        <v>911715</v>
       </c>
       <c r="P691" s="6">
         <v>58498</v>
@@ -57147,10 +57150,10 @@
         <v>78</v>
       </c>
       <c r="S691" s="6">
-        <v>974585</v>
+        <v>974980</v>
       </c>
       <c r="T691" s="6">
-        <v>530583</v>
+        <v>530648</v>
       </c>
       <c r="U691" s="6">
         <v>60129</v>
@@ -57162,10 +57165,10 @@
         <v>108</v>
       </c>
       <c r="X691" s="6">
-        <v>594400</v>
+        <v>594465</v>
       </c>
       <c r="Y691" s="6">
-        <v>1568985</v>
+        <v>1569445</v>
       </c>
     </row>
     <row r="692" spans="1:25" x14ac:dyDescent="0.25">
@@ -57188,31 +57191,31 @@
         <v>937765</v>
       </c>
       <c r="G692" s="6">
-        <v>10681</v>
+        <v>12002</v>
       </c>
       <c r="H692" s="6">
-        <v>948446</v>
+        <v>949767</v>
       </c>
       <c r="I692" s="6">
         <v>445313</v>
       </c>
       <c r="J692" s="6">
-        <v>15559</v>
+        <v>15527</v>
       </c>
       <c r="K692" s="6">
-        <v>460872</v>
+        <v>460840</v>
       </c>
       <c r="L692" s="6">
         <v>1383078</v>
       </c>
       <c r="M692" s="6">
-        <v>26240</v>
+        <v>27529</v>
       </c>
       <c r="N692" s="6">
-        <v>1409318</v>
+        <v>1410607</v>
       </c>
       <c r="O692" s="6">
-        <v>884230</v>
+        <v>885551</v>
       </c>
       <c r="P692" s="6">
         <v>61516</v>
@@ -57224,13 +57227,13 @@
         <v>22</v>
       </c>
       <c r="S692" s="6">
-        <v>948446</v>
+        <v>949767</v>
       </c>
       <c r="T692" s="6">
         <v>405590</v>
       </c>
       <c r="U692" s="6">
-        <v>52515</v>
+        <v>52483</v>
       </c>
       <c r="V692" s="6">
         <v>2697</v>
@@ -57239,10 +57242,10 @@
         <v>70</v>
       </c>
       <c r="X692" s="6">
-        <v>460872</v>
+        <v>460840</v>
       </c>
       <c r="Y692" s="6">
-        <v>1409318</v>
+        <v>1410607</v>
       </c>
     </row>
     <row r="693" spans="1:25" x14ac:dyDescent="0.25">
@@ -57265,31 +57268,31 @@
         <v>800679</v>
       </c>
       <c r="G693" s="6">
-        <v>56421</v>
+        <v>51711</v>
       </c>
       <c r="H693" s="6">
-        <v>857100</v>
+        <v>852390</v>
       </c>
       <c r="I693" s="6">
         <v>343793</v>
       </c>
       <c r="J693" s="6">
-        <v>75807</v>
+        <v>76033</v>
       </c>
       <c r="K693" s="6">
-        <v>419600</v>
+        <v>419826</v>
       </c>
       <c r="L693" s="6">
         <v>1144472</v>
       </c>
       <c r="M693" s="6">
-        <v>132228</v>
+        <v>127744</v>
       </c>
       <c r="N693" s="6">
-        <v>1276700</v>
+        <v>1272216</v>
       </c>
       <c r="O693" s="6">
-        <v>791163</v>
+        <v>786453</v>
       </c>
       <c r="P693" s="6">
         <v>62303</v>
@@ -57301,10 +57304,10 @@
         <v>6</v>
       </c>
       <c r="S693" s="6">
-        <v>857100</v>
+        <v>852390</v>
       </c>
       <c r="T693" s="6">
-        <v>378007</v>
+        <v>378233</v>
       </c>
       <c r="U693" s="6">
         <v>40682</v>
@@ -57316,10 +57319,10 @@
         <v>24</v>
       </c>
       <c r="X693" s="6">
-        <v>419600</v>
+        <v>419826</v>
       </c>
       <c r="Y693" s="6">
-        <v>1276700</v>
+        <v>1272216</v>
       </c>
     </row>
     <row r="694" spans="1:25" x14ac:dyDescent="0.25">
@@ -57419,31 +57422,31 @@
         <v>268544</v>
       </c>
       <c r="G695" s="6">
-        <v>618</v>
+        <v>991</v>
       </c>
       <c r="H695" s="6">
-        <v>269162</v>
+        <v>269535</v>
       </c>
       <c r="I695" s="6">
         <v>85485</v>
       </c>
       <c r="J695" s="6">
-        <v>1070</v>
+        <v>2628</v>
       </c>
       <c r="K695" s="6">
-        <v>86555</v>
+        <v>88113</v>
       </c>
       <c r="L695" s="6">
         <v>354029</v>
       </c>
       <c r="M695" s="6">
-        <v>1688</v>
+        <v>3619</v>
       </c>
       <c r="N695" s="6">
-        <v>355717</v>
+        <v>357648</v>
       </c>
       <c r="O695" s="6">
-        <v>237149</v>
+        <v>237522</v>
       </c>
       <c r="P695" s="6">
         <v>30086</v>
@@ -57455,13 +57458,13 @@
         <v>4</v>
       </c>
       <c r="S695" s="6">
-        <v>269162</v>
+        <v>269535</v>
       </c>
       <c r="T695" s="6">
-        <v>80033</v>
+        <v>80880</v>
       </c>
       <c r="U695" s="6">
-        <v>6132</v>
+        <v>6843</v>
       </c>
       <c r="V695" s="6">
         <v>86</v>
@@ -57470,10 +57473,10 @@
         <v>304</v>
       </c>
       <c r="X695" s="6">
-        <v>86555</v>
+        <v>88113</v>
       </c>
       <c r="Y695" s="6">
-        <v>355717</v>
+        <v>357648</v>
       </c>
     </row>
     <row r="696" spans="1:25" x14ac:dyDescent="0.25">
@@ -57483,7 +57486,7 @@
       <c r="B696" s="4">
         <v>25</v>
       </c>
-      <c r="C696" s="60" t="s">
+      <c r="C696" s="59" t="s">
         <v>737</v>
       </c>
       <c r="D696" s="6" t="s">
@@ -57496,31 +57499,31 @@
         <v>432804</v>
       </c>
       <c r="G696" s="6">
-        <v>0</v>
+        <v>-5334</v>
       </c>
       <c r="H696" s="6">
-        <v>432804</v>
+        <v>427470</v>
       </c>
       <c r="I696" s="6">
         <v>150038</v>
       </c>
       <c r="J696" s="6">
-        <v>0</v>
+        <v>1140</v>
       </c>
       <c r="K696" s="6">
-        <v>150038</v>
+        <v>151178</v>
       </c>
       <c r="L696" s="6">
         <v>582842</v>
       </c>
       <c r="M696" s="6">
-        <v>0</v>
+        <v>-4194</v>
       </c>
       <c r="N696" s="6">
-        <v>582842</v>
+        <v>578648</v>
       </c>
       <c r="O696" s="6">
-        <v>379826</v>
+        <v>374492</v>
       </c>
       <c r="P696" s="6">
         <v>48627</v>
@@ -57532,10 +57535,10 @@
         <v>28</v>
       </c>
       <c r="S696" s="6">
-        <v>432804</v>
+        <v>427470</v>
       </c>
       <c r="T696" s="6">
-        <v>134150</v>
+        <v>135290</v>
       </c>
       <c r="U696" s="6">
         <v>15007</v>
@@ -57547,10 +57550,10 @@
         <v>7</v>
       </c>
       <c r="X696" s="6">
-        <v>150038</v>
+        <v>151178</v>
       </c>
       <c r="Y696" s="6">
-        <v>582842</v>
+        <v>578648</v>
       </c>
     </row>
     <row r="697" spans="1:25" x14ac:dyDescent="0.25">
@@ -57560,33 +57563,75 @@
       <c r="B697" s="4">
         <v>26</v>
       </c>
-      <c r="C697" s="7"/>
+      <c r="C697" s="60" t="s">
+        <v>738</v>
+      </c>
       <c r="D697" s="6" t="s">
         <v>77</v>
       </c>
       <c r="E697" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F697" s="6"/>
-      <c r="G697" s="6"/>
-      <c r="H697" s="6"/>
-      <c r="I697" s="6"/>
-      <c r="J697" s="6"/>
-      <c r="K697" s="6"/>
-      <c r="L697" s="6"/>
-      <c r="M697" s="6"/>
-      <c r="N697" s="6"/>
-      <c r="O697" s="6"/>
-      <c r="P697" s="6"/>
-      <c r="Q697" s="6"/>
-      <c r="R697" s="6"/>
-      <c r="S697" s="6"/>
-      <c r="T697" s="6"/>
-      <c r="U697" s="6"/>
-      <c r="V697" s="6"/>
-      <c r="W697" s="6"/>
-      <c r="X697" s="6"/>
-      <c r="Y697" s="6"/>
+      <c r="F697" s="6">
+        <v>260568</v>
+      </c>
+      <c r="G697" s="6">
+        <v>0</v>
+      </c>
+      <c r="H697" s="6">
+        <v>260568</v>
+      </c>
+      <c r="I697" s="6">
+        <v>109681</v>
+      </c>
+      <c r="J697" s="6">
+        <v>0</v>
+      </c>
+      <c r="K697" s="6">
+        <v>109681</v>
+      </c>
+      <c r="L697" s="6">
+        <v>370249</v>
+      </c>
+      <c r="M697" s="6">
+        <v>0</v>
+      </c>
+      <c r="N697" s="6">
+        <v>370249</v>
+      </c>
+      <c r="O697" s="6">
+        <v>230737</v>
+      </c>
+      <c r="P697" s="6">
+        <v>26757</v>
+      </c>
+      <c r="Q697" s="6">
+        <v>3065</v>
+      </c>
+      <c r="R697" s="6">
+        <v>9</v>
+      </c>
+      <c r="S697" s="6">
+        <v>260568</v>
+      </c>
+      <c r="T697" s="6">
+        <v>101143</v>
+      </c>
+      <c r="U697" s="6">
+        <v>8174</v>
+      </c>
+      <c r="V697" s="6">
+        <v>304</v>
+      </c>
+      <c r="W697" s="6">
+        <v>60</v>
+      </c>
+      <c r="X697" s="6">
+        <v>109681</v>
+      </c>
+      <c r="Y697" s="6">
+        <v>370249</v>
+      </c>
     </row>
     <row r="698" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A698" s="7">
@@ -58768,17 +58813,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010075ECE796D7EABA42BC0DB2CA73C7CE00" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e2ecee1b3d34a959aed38d5dc4c878f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8" xmlns:ns3="ae149517-eeaa-465d-b3b6-396a1e23bc6e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9af26d9f7c79c0f2a842447557dfee25" ns2:_="" ns3:_="">
     <xsd:import namespace="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
@@ -59005,6 +59039,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ae149517-eeaa-465d-b3b6-396a1e23bc6e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -59015,17 +59060,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
-    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A42C790-3343-4FC1-9ABA-46A7C5CDBF94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -59044,6 +59078,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B269C13-F95E-434A-9E7B-CE8B41B5A4E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ae149517-eeaa-465d-b3b6-396a1e23bc6e"/>
+    <ds:schemaRef ds:uri="3fe4ae0e-3af2-48f1-b2fd-da4a302e5eb8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B35FBC-7726-46DC-BCFD-4B2C0893BC60}">
   <ds:schemaRefs>

</xml_diff>